<commit_message>
docs: update Zenodo catalog through intake batch 6
Add the audited 59-file / 45-work intake checkpoint, evidence gates, and protected-material boundaries without publishing private source documents.
</commit_message>
<xml_diff>
--- a/docs/portfolio/zenodo/Mya_Brown_Zenodo_Master_Catalog_and_Development_Pipeline.xlsx
+++ b/docs/portfolio/zenodo/Mya_Brown_Zenodo_Master_Catalog_and_Development_Pipeline.xlsx
@@ -2,11 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="R3166c9b5842445b4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Master Catalog" sheetId="2" r:id="R30616ea13eda42dd"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Development Pipeline" sheetId="3" r:id="R84944529e244423d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Validation &amp; Partners" sheetId="4" r:id="R36c5e5a5ebe548ed"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="5" r:id="Rdf908f8642364056"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="R9c507850fd004a40"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Master Catalog" sheetId="2" r:id="R8beffc184cd14c5f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Development Pipeline" sheetId="3" r:id="R5b87a5335f7749ed"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Validation &amp; Partners" sheetId="4" r:id="Rc61dd578c0bd4ee2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="5" r:id="R64c0758339004c8e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Document Intake" sheetId="6" r:id="R11830168a2bb4fa7"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -60,7 +61,7 @@
       <x:name val="Arial"/>
     </x:font>
   </x:fonts>
-  <x:fills count="7">
+  <x:fills count="8">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -92,8 +93,13 @@
         <x:fgColor rgb="FF595959"/>
       </x:patternFill>
     </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF60497A"/>
+      </x:patternFill>
+    </x:fill>
   </x:fills>
-  <x:borders count="6">
+  <x:borders count="9">
     <x:border/>
     <x:border>
       <x:left style="thin">
@@ -138,11 +144,32 @@
         <x:color rgb="FFB4C7E7"/>
       </x:bottom>
     </x:border>
+    <x:border>
+      <x:bottom style="thin">
+        <x:color rgb="FFD9D2E9"/>
+      </x:bottom>
+    </x:border>
+    <x:border>
+      <x:top style="thin">
+        <x:color rgb="FFD9D2E9"/>
+      </x:top>
+      <x:bottom style="thin">
+        <x:color rgb="FFD9D2E9"/>
+      </x:bottom>
+    </x:border>
+    <x:border>
+      <x:top style="thin">
+        <x:color rgb="FFD9D2E9"/>
+      </x:top>
+      <x:bottom style="thin">
+        <x:color rgb="FFB1A0C7"/>
+      </x:bottom>
+    </x:border>
   </x:borders>
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="47">
+  <x:cellXfs count="53">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -247,6 +274,20 @@
     <x:xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="top" wrapText="1"/>
     </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="2" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="2" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="2" fillId="7" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
     <x:xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center" wrapText="1"/>
     </x:xf>
@@ -320,6 +361,20 @@
     <x:tableColumn id="5" name="Limitation"/>
   </x:tableColumns>
   <x:tableStyleInfo name="TableStyleMedium3" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</x:table>
+</file>
+
+<file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="DocumentIntake" displayName="DocumentIntake" ref="A1:F60" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:tableColumns count="6">
+    <x:tableColumn id="1" name="Source document"/>
+    <x:tableColumn id="2" name="Portfolio type"/>
+    <x:tableColumn id="3" name="Release disposition"/>
+    <x:tableColumn id="4" name="Zenodo match status"/>
+    <x:tableColumn id="5" name="Working description"/>
+    <x:tableColumn id="6" name="Next evidence gate"/>
+  </x:tableColumns>
+  <x:tableStyleInfo name="TableStyleMedium4" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </x:table>
 </file>
 
@@ -532,14 +587,14 @@
   </x:cols>
   <x:sheetData>
     <x:row r="1">
-      <x:c r="A1" s="46"/>
-      <x:c r="B1" s="46"/>
-      <x:c r="C1" s="46"/>
-      <x:c r="D1" s="46"/>
-      <x:c r="E1" s="46"/>
-      <x:c r="F1" s="46"/>
-      <x:c r="G1" s="46"/>
-      <x:c r="H1" s="46"/>
+      <x:c r="A1" s="52"/>
+      <x:c r="B1" s="52"/>
+      <x:c r="C1" s="52"/>
+      <x:c r="D1" s="52"/>
+      <x:c r="E1" s="52"/>
+      <x:c r="F1" s="52"/>
+      <x:c r="G1" s="52"/>
+      <x:c r="H1" s="52"/>
     </x:row>
     <x:row r="2">
       <x:c r="A2" s="21" t="str">
@@ -554,14 +609,14 @@
       <x:c r="H2" s="21"/>
     </x:row>
     <x:row r="3">
-      <x:c r="A3" s="46"/>
-      <x:c r="B3" s="46"/>
-      <x:c r="C3" s="46"/>
-      <x:c r="D3" s="46"/>
-      <x:c r="E3" s="46"/>
-      <x:c r="F3" s="46"/>
-      <x:c r="G3" s="46"/>
-      <x:c r="H3" s="46"/>
+      <x:c r="A3" s="52"/>
+      <x:c r="B3" s="52"/>
+      <x:c r="C3" s="52"/>
+      <x:c r="D3" s="52"/>
+      <x:c r="E3" s="52"/>
+      <x:c r="F3" s="52"/>
+      <x:c r="G3" s="52"/>
+      <x:c r="H3" s="52"/>
     </x:row>
     <x:row r="4">
       <x:c r="A4" s="22" t="str">
@@ -570,12 +625,12 @@
       <x:c r="B4" s="23" t="str">
         <x:v>Value</x:v>
       </x:c>
-      <x:c r="C4" s="46"/>
-      <x:c r="D4" s="46"/>
-      <x:c r="E4" s="46"/>
-      <x:c r="F4" s="46"/>
-      <x:c r="G4" s="46"/>
-      <x:c r="H4" s="46"/>
+      <x:c r="C4" s="52"/>
+      <x:c r="D4" s="52"/>
+      <x:c r="E4" s="52"/>
+      <x:c r="F4" s="52"/>
+      <x:c r="G4" s="52"/>
+      <x:c r="H4" s="52"/>
     </x:row>
     <x:row r="5">
       <x:c r="A5" s="24" t="str">
@@ -584,40 +639,40 @@
       <x:c r="B5" s="24" t="n">
         <x:v>60</x:v>
       </x:c>
-      <x:c r="C5" s="46"/>
-      <x:c r="D5" s="46"/>
-      <x:c r="E5" s="46"/>
-      <x:c r="F5" s="46"/>
-      <x:c r="G5" s="46"/>
-      <x:c r="H5" s="46"/>
+      <x:c r="C5" s="52"/>
+      <x:c r="D5" s="52"/>
+      <x:c r="E5" s="52"/>
+      <x:c r="F5" s="52"/>
+      <x:c r="G5" s="52"/>
+      <x:c r="H5" s="52"/>
     </x:row>
     <x:row r="6">
       <x:c r="A6" s="24" t="str">
-        <x:v>Total results shown in preserved captures</x:v>
+        <x:v>Local source files / unique works</x:v>
       </x:c>
       <x:c r="B6" s="24" t="str">
-        <x:v>262–272</x:v>
-      </x:c>
-      <x:c r="C6" s="46"/>
-      <x:c r="D6" s="46"/>
-      <x:c r="E6" s="46"/>
-      <x:c r="F6" s="46"/>
-      <x:c r="G6" s="46"/>
-      <x:c r="H6" s="46"/>
+        <x:v>59 files / 45 unique</x:v>
+      </x:c>
+      <x:c r="C6" s="52"/>
+      <x:c r="D6" s="52"/>
+      <x:c r="E6" s="52"/>
+      <x:c r="F6" s="52"/>
+      <x:c r="G6" s="52"/>
+      <x:c r="H6" s="52"/>
     </x:row>
     <x:row r="7">
       <x:c r="A7" s="24" t="str">
-        <x:v>Unrecovered record gap</x:v>
+        <x:v>Total / gap shown in preserved captures</x:v>
       </x:c>
       <x:c r="B7" s="24" t="str">
-        <x:v>202–212</x:v>
-      </x:c>
-      <x:c r="C7" s="46"/>
-      <x:c r="D7" s="46"/>
-      <x:c r="E7" s="46"/>
-      <x:c r="F7" s="46"/>
-      <x:c r="G7" s="46"/>
-      <x:c r="H7" s="46"/>
+        <x:v>262–272 total / 202–212 unrecovered</x:v>
+      </x:c>
+      <x:c r="C7" s="52"/>
+      <x:c r="D7" s="52"/>
+      <x:c r="E7" s="52"/>
+      <x:c r="F7" s="52"/>
+      <x:c r="G7" s="52"/>
+      <x:c r="H7" s="52"/>
     </x:row>
     <x:row r="8">
       <x:c r="A8" s="24" t="str">
@@ -626,12 +681,12 @@
       <x:c r="B8" s="24" t="str">
         <x:v>Mya P. Brown — Commons Initiative</x:v>
       </x:c>
-      <x:c r="C8" s="46"/>
-      <x:c r="D8" s="46"/>
-      <x:c r="E8" s="46"/>
-      <x:c r="F8" s="46"/>
-      <x:c r="G8" s="46"/>
-      <x:c r="H8" s="46"/>
+      <x:c r="C8" s="52"/>
+      <x:c r="D8" s="52"/>
+      <x:c r="E8" s="52"/>
+      <x:c r="F8" s="52"/>
+      <x:c r="G8" s="52"/>
+      <x:c r="H8" s="52"/>
     </x:row>
     <x:row r="9">
       <x:c r="A9" s="24" t="str">
@@ -640,12 +695,12 @@
       <x:c r="B9" s="25" t="n">
         <x:v>46283</x:v>
       </x:c>
-      <x:c r="C9" s="46"/>
-      <x:c r="D9" s="46"/>
-      <x:c r="E9" s="46"/>
-      <x:c r="F9" s="46"/>
-      <x:c r="G9" s="46"/>
-      <x:c r="H9" s="46"/>
+      <x:c r="C9" s="52"/>
+      <x:c r="D9" s="52"/>
+      <x:c r="E9" s="52"/>
+      <x:c r="F9" s="52"/>
+      <x:c r="G9" s="52"/>
+      <x:c r="H9" s="52"/>
     </x:row>
     <x:row r="10">
       <x:c r="A10" s="24" t="str">
@@ -654,22 +709,22 @@
       <x:c r="B10" s="24" t="str">
         <x:v>Publication or DOI proves provenance, not scientific validation or market readiness.</x:v>
       </x:c>
-      <x:c r="C10" s="46"/>
-      <x:c r="D10" s="46"/>
-      <x:c r="E10" s="46"/>
-      <x:c r="F10" s="46"/>
-      <x:c r="G10" s="46"/>
-      <x:c r="H10" s="46"/>
+      <x:c r="C10" s="52"/>
+      <x:c r="D10" s="52"/>
+      <x:c r="E10" s="52"/>
+      <x:c r="F10" s="52"/>
+      <x:c r="G10" s="52"/>
+      <x:c r="H10" s="52"/>
     </x:row>
     <x:row r="11">
-      <x:c r="A11" s="46"/>
-      <x:c r="B11" s="46"/>
-      <x:c r="C11" s="46"/>
-      <x:c r="D11" s="46"/>
-      <x:c r="E11" s="46"/>
-      <x:c r="F11" s="46"/>
-      <x:c r="G11" s="46"/>
-      <x:c r="H11" s="46"/>
+      <x:c r="A11" s="52"/>
+      <x:c r="B11" s="52"/>
+      <x:c r="C11" s="52"/>
+      <x:c r="D11" s="52"/>
+      <x:c r="E11" s="52"/>
+      <x:c r="F11" s="52"/>
+      <x:c r="G11" s="52"/>
+      <x:c r="H11" s="52"/>
     </x:row>
     <x:row r="12">
       <x:c r="A12" s="26" t="str">
@@ -684,10 +739,10 @@
       <x:c r="D12" s="26" t="str">
         <x:v>Gate</x:v>
       </x:c>
-      <x:c r="E12" s="46"/>
-      <x:c r="F12" s="46"/>
-      <x:c r="G12" s="46"/>
-      <x:c r="H12" s="46"/>
+      <x:c r="E12" s="52"/>
+      <x:c r="F12" s="52"/>
+      <x:c r="G12" s="52"/>
+      <x:c r="H12" s="52"/>
     </x:row>
     <x:row r="13">
       <x:c r="A13" s="24" t="n">
@@ -702,10 +757,10 @@
       <x:c r="D13" s="24" t="str">
         <x:v>Deliver to first 3 clients; record correction and consent path</x:v>
       </x:c>
-      <x:c r="E13" s="46"/>
-      <x:c r="F13" s="46"/>
-      <x:c r="G13" s="46"/>
-      <x:c r="H13" s="46"/>
+      <x:c r="E13" s="52"/>
+      <x:c r="F13" s="52"/>
+      <x:c r="G13" s="52"/>
+      <x:c r="H13" s="52"/>
     </x:row>
     <x:row r="14">
       <x:c r="A14" s="24" t="n">
@@ -720,10 +775,10 @@
       <x:c r="D14" s="24" t="str">
         <x:v>Passing deterministic tests; permissions and rollback visible</x:v>
       </x:c>
-      <x:c r="E14" s="46"/>
-      <x:c r="F14" s="46"/>
-      <x:c r="G14" s="46"/>
-      <x:c r="H14" s="46"/>
+      <x:c r="E14" s="52"/>
+      <x:c r="F14" s="52"/>
+      <x:c r="G14" s="52"/>
+      <x:c r="H14" s="52"/>
     </x:row>
     <x:row r="15">
       <x:c r="A15" s="24" t="n">
@@ -738,10 +793,10 @@
       <x:c r="D15" s="24" t="str">
         <x:v>No physical product claim until working prototype and safety review</x:v>
       </x:c>
-      <x:c r="E15" s="46"/>
-      <x:c r="F15" s="46"/>
-      <x:c r="G15" s="46"/>
-      <x:c r="H15" s="46"/>
+      <x:c r="E15" s="52"/>
+      <x:c r="F15" s="52"/>
+      <x:c r="G15" s="52"/>
+      <x:c r="H15" s="52"/>
     </x:row>
     <x:row r="16">
       <x:c r="A16" s="24" t="n">
@@ -756,10 +811,10 @@
       <x:c r="D16" s="24" t="str">
         <x:v>Repeatable data on speed, shape, tension, and failure modes</x:v>
       </x:c>
-      <x:c r="E16" s="46"/>
-      <x:c r="F16" s="46"/>
-      <x:c r="G16" s="46"/>
-      <x:c r="H16" s="46"/>
+      <x:c r="E16" s="52"/>
+      <x:c r="F16" s="52"/>
+      <x:c r="G16" s="52"/>
+      <x:c r="H16" s="52"/>
     </x:row>
     <x:row r="17">
       <x:c r="A17" s="24" t="n">
@@ -774,10 +829,10 @@
       <x:c r="D17" s="24" t="str">
         <x:v>Independent aerospace review; no geoengineering claim</x:v>
       </x:c>
-      <x:c r="E17" s="46"/>
-      <x:c r="F17" s="46"/>
-      <x:c r="G17" s="46"/>
-      <x:c r="H17" s="46"/>
+      <x:c r="E17" s="52"/>
+      <x:c r="F17" s="52"/>
+      <x:c r="G17" s="52"/>
+      <x:c r="H17" s="52"/>
     </x:row>
     <x:row r="18">
       <x:c r="A18" s="24" t="n">
@@ -792,20 +847,20 @@
       <x:c r="D18" s="24" t="str">
         <x:v>No wet-lab or human work without qualified partners and approvals</x:v>
       </x:c>
-      <x:c r="E18" s="46"/>
-      <x:c r="F18" s="46"/>
-      <x:c r="G18" s="46"/>
-      <x:c r="H18" s="46"/>
+      <x:c r="E18" s="52"/>
+      <x:c r="F18" s="52"/>
+      <x:c r="G18" s="52"/>
+      <x:c r="H18" s="52"/>
     </x:row>
     <x:row r="19">
-      <x:c r="A19" s="46"/>
-      <x:c r="B19" s="46"/>
-      <x:c r="C19" s="46"/>
-      <x:c r="D19" s="46"/>
-      <x:c r="E19" s="46"/>
-      <x:c r="F19" s="46"/>
-      <x:c r="G19" s="46"/>
-      <x:c r="H19" s="46"/>
+      <x:c r="A19" s="52"/>
+      <x:c r="B19" s="52"/>
+      <x:c r="C19" s="52"/>
+      <x:c r="D19" s="52"/>
+      <x:c r="E19" s="52"/>
+      <x:c r="F19" s="52"/>
+      <x:c r="G19" s="52"/>
+      <x:c r="H19" s="52"/>
     </x:row>
     <x:row r="20">
       <x:c r="A20" s="27" t="str">
@@ -912,24 +967,24 @@
       </x:c>
     </x:row>
     <x:row r="24">
-      <x:c r="A24" s="46"/>
-      <x:c r="B24" s="46"/>
-      <x:c r="C24" s="46"/>
-      <x:c r="D24" s="46"/>
-      <x:c r="E24" s="46"/>
-      <x:c r="F24" s="46"/>
-      <x:c r="G24" s="46"/>
-      <x:c r="H24" s="46"/>
+      <x:c r="A24" s="52"/>
+      <x:c r="B24" s="52"/>
+      <x:c r="C24" s="52"/>
+      <x:c r="D24" s="52"/>
+      <x:c r="E24" s="52"/>
+      <x:c r="F24" s="52"/>
+      <x:c r="G24" s="52"/>
+      <x:c r="H24" s="52"/>
     </x:row>
     <x:row r="25">
-      <x:c r="A25" s="46"/>
-      <x:c r="B25" s="46"/>
-      <x:c r="C25" s="46"/>
-      <x:c r="D25" s="46"/>
-      <x:c r="E25" s="46"/>
-      <x:c r="F25" s="46"/>
-      <x:c r="G25" s="46"/>
-      <x:c r="H25" s="46"/>
+      <x:c r="A25" s="52"/>
+      <x:c r="B25" s="52"/>
+      <x:c r="C25" s="52"/>
+      <x:c r="D25" s="52"/>
+      <x:c r="E25" s="52"/>
+      <x:c r="F25" s="52"/>
+      <x:c r="G25" s="52"/>
+      <x:c r="H25" s="52"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -3281,7 +3336,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6d14e26f1dbb4dc8"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf59d0a835c92418f"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4612,7 +4667,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6838a5ff9e834751"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R07b416a7f00148a3"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4871,7 +4926,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb3c1ebce56124b00"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra5ed2f2eba674c70"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5063,7 +5118,1230 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rece124d4f5c94c12"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf9b28abd347a4872"/>
+  </x:tableParts>
+</x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetPr>
+    <x:tabColor rgb="FF8064A2"/>
+  </x:sheetPr>
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="52" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="34" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="34" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="28" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="70" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="76" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1">
+      <x:c r="A1" s="49" t="str">
+        <x:v>Source document</x:v>
+      </x:c>
+      <x:c r="B1" s="49" t="str">
+        <x:v>Portfolio type</x:v>
+      </x:c>
+      <x:c r="C1" s="49" t="str">
+        <x:v>Release disposition</x:v>
+      </x:c>
+      <x:c r="D1" s="49" t="str">
+        <x:v>Zenodo match status</x:v>
+      </x:c>
+      <x:c r="E1" s="49" t="str">
+        <x:v>Working description</x:v>
+      </x:c>
+      <x:c r="F1" s="49" t="str">
+        <x:v>Next evidence gate</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2">
+      <x:c r="A2" s="50" t="str">
+        <x:v>Civilizational Maturity and the Collision Prevention Principle</x:v>
+      </x:c>
+      <x:c r="B2" s="50" t="str">
+        <x:v>Conceptual research paper / systems governance</x:v>
+      </x:c>
+      <x:c r="C2" s="50" t="str">
+        <x:v>Public candidate</x:v>
+      </x:c>
+      <x:c r="D2" s="50" t="str">
+        <x:v>No match in recovered 60</x:v>
+      </x:c>
+      <x:c r="E2" s="50" t="str">
+        <x:v>Civilizational-risk framework linking capability, restraint, collision prevention, material security, and lifelong education.</x:v>
+      </x:c>
+      <x:c r="F2" s="50" t="str">
+        <x:v>Normalize citations and claims; attach CERL; final PDF; independent subject-matter and legal review.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="3">
+      <x:c r="A3" s="50" t="str">
+        <x:v>From Continuity-Governed AI to Adversarially Governed Technology</x:v>
+      </x:c>
+      <x:c r="B3" s="50" t="str">
+        <x:v>Research update / technical note</x:v>
+      </x:c>
+      <x:c r="C3" s="50" t="str">
+        <x:v>Public candidate</x:v>
+      </x:c>
+      <x:c r="D3" s="50" t="str">
+        <x:v>No match in recovered 60</x:v>
+      </x:c>
+      <x:c r="E3" s="50" t="str">
+        <x:v>Integration lessons across Commons Sentience Sandbox, MAYA Node, SAGE, CERL-Preemptive, and Commons governance.</x:v>
+      </x:c>
+      <x:c r="F3" s="50" t="str">
+        <x:v>Repair citation artifacts; verify implementation claims; add evidence labels; independent security/governance review.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="4">
+      <x:c r="A4" s="50" t="str">
+        <x:v>The Pathology of Unaccountable Power</x:v>
+      </x:c>
+      <x:c r="B4" s="50" t="str">
+        <x:v>Research and governance paper</x:v>
+      </x:c>
+      <x:c r="C4" s="50" t="str">
+        <x:v>Public candidate after source audit</x:v>
+      </x:c>
+      <x:c r="D4" s="50" t="str">
+        <x:v>No match in recovered 60</x:v>
+      </x:c>
+      <x:c r="E4" s="50" t="str">
+        <x:v>Adversarial-governance argument with an evidence file of institutional abuse, concealment, and failure cases.</x:v>
+      </x:c>
+      <x:c r="F4" s="50" t="str">
+        <x:v>Audit every factual claim and citation; separate evidence from inference; add safeguard counter-cases; external review.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5">
+      <x:c r="A5" s="50" t="str">
+        <x:v>The Blue Book: Systems Accountability Engineering</x:v>
+      </x:c>
+      <x:c r="B5" s="50" t="str">
+        <x:v>Governance and engineering framework</x:v>
+      </x:c>
+      <x:c r="C5" s="50" t="str">
+        <x:v>Public candidate after editorial review</x:v>
+      </x:c>
+      <x:c r="D5" s="50" t="str">
+        <x:v>No match in recovered 60</x:v>
+      </x:c>
+      <x:c r="E5" s="50" t="str">
+        <x:v>Refined SAE framework for outcomes, failure resilience, accountability, correction, rights, and succession.</x:v>
+      </x:c>
+      <x:c r="F5" s="50" t="str">
+        <x:v>Use as canonical candidate; reconcile citations, version and license; remove conversational residue; technical/legal/editorial review.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6">
+      <x:c r="A6" s="50" t="str">
+        <x:v>The Blue Book: A Systems Accountability Engineering Framework for Building Things That Actually Work</x:v>
+      </x:c>
+      <x:c r="B6" s="50" t="str">
+        <x:v>Earlier working draft / duplicate lineage</x:v>
+      </x:c>
+      <x:c r="C6" s="50" t="str">
+        <x:v>Private working source</x:v>
+      </x:c>
+      <x:c r="D6" s="50" t="str">
+        <x:v>Related duplicate lineage</x:v>
+      </x:c>
+      <x:c r="E6" s="50" t="str">
+        <x:v>Earlier conversational draft containing the core questions, lifecycle loop, accountability layer, and fictional-character tests.</x:v>
+      </x:c>
+      <x:c r="F6" s="50" t="str">
+        <x:v>Diff against refined Blue Book; preserve unique material in version history; do not release as independent work without lineage note.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7">
+      <x:c r="A7" s="50" t="str">
+        <x:v>Titan-Grip Brake Project — Engineering Handoff DR-01 / Pre-Level-0.5</x:v>
+      </x:c>
+      <x:c r="B7" s="50" t="str">
+        <x:v>Invention / mechanical engineering development</x:v>
+      </x:c>
+      <x:c r="C7" s="50" t="str">
+        <x:v>Private technical development</x:v>
+      </x:c>
+      <x:c r="D7" s="50" t="str">
+        <x:v>No match in recovered 60</x:v>
+      </x:c>
+      <x:c r="E7" s="50" t="str">
+        <x:v>Brake-system investigation covering physical evidence, failure hypotheses, baseline tests, and candidate architectures.</x:v>
+      </x:c>
+      <x:c r="F7" s="50" t="str">
+        <x:v>Keep design details private; complete corrected-system baseline and calibrated measurements; independent brake/test-safety review.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8">
+      <x:c r="A8" s="50" t="str">
+        <x:v>The Queen AE86 — Royal Blue Book, Vehicle No. 086</x:v>
+      </x:c>
+      <x:c r="B8" s="50" t="str">
+        <x:v>Vehicle restoration and build manual</x:v>
+      </x:c>
+      <x:c r="C8" s="50" t="str">
+        <x:v>Private working publication</x:v>
+      </x:c>
+      <x:c r="D8" s="50" t="str">
+        <x:v>No match in recovered 60</x:v>
+      </x:c>
+      <x:c r="E8" s="50" t="str">
+        <x:v>Toyota AE86 history, inspection, restoration, modification, safety, maintenance, and build-record book.</x:v>
+      </x:c>
+      <x:c r="F8" s="50" t="str">
+        <x:v>Verify specifications; add chassis/market caveats; trademark, safety, rights, and editorial review.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9">
+      <x:c r="A9" s="50" t="str">
+        <x:v>Starfleet Academy — San Francisco Campus</x:v>
+      </x:c>
+      <x:c r="B9" s="50" t="str">
+        <x:v>Fiction-based curriculum / interactive learning program</x:v>
+      </x:c>
+      <x:c r="C9" s="50" t="str">
+        <x:v>Rights-restricted working source</x:v>
+      </x:c>
+      <x:c r="D9" s="50" t="str">
+        <x:v>No match in recovered 60</x:v>
+      </x:c>
+      <x:c r="E9" s="50" t="str">
+        <x:v>Four-year Starfleet-inspired cadet curriculum with daily orders, classes, simulations, and evaluations.</x:v>
+      </x:c>
+      <x:c r="F9" s="50" t="str">
+        <x:v>Do not present as official; separate original pedagogy from third-party IP or create a rights-cleared original academy.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10">
+      <x:c r="A10" s="50" t="str">
+        <x:v>The Gotham Anomaly Archive — Recovered Research Edition</x:v>
+      </x:c>
+      <x:c r="B10" s="50" t="str">
+        <x:v>Transformative fan scholarship and original fiction</x:v>
+      </x:c>
+      <x:c r="C10" s="50" t="str">
+        <x:v>Rights-restricted publication candidate</x:v>
+      </x:c>
+      <x:c r="D10" s="50" t="str">
+        <x:v>No match in recovered 60</x:v>
+      </x:c>
+      <x:c r="E10" s="50" t="str">
+        <x:v>75-page continuity-aware Gotham dossier and documentary-horror narrative with an unofficial fan-scholarship notice.</x:v>
+      </x:c>
+      <x:c r="F10" s="50" t="str">
+        <x:v>Keep full PDF out of public GitHub; citation, quotation, image, trademark, accessibility, and distribution review.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11">
+      <x:c r="A11" s="50" t="str">
+        <x:v>The Cost of the Foundation</x:v>
+      </x:c>
+      <x:c r="B11" s="50" t="str">
+        <x:v>Historical and reparations essay / working manuscript</x:v>
+      </x:c>
+      <x:c r="C11" s="50" t="str">
+        <x:v>Private until evidence and editorial review</x:v>
+      </x:c>
+      <x:c r="D11" s="50" t="str">
+        <x:v>No match in recovered 60</x:v>
+      </x:c>
+      <x:c r="E11" s="50" t="str">
+        <x:v>Working essay on the slave trade, African-American history, reparations, institutional resistance, and human development.</x:v>
+      </x:c>
+      <x:c r="F11" s="50" t="str">
+        <x:v>Consolidate repeated drafts; ground claims in primary/scholarly sources; Black-studies, African-history, legal, and sensitivity review.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12">
+      <x:c r="A12" s="50" t="str">
+        <x:v>260701_CP Brown_STMT</x:v>
+      </x:c>
+      <x:c r="B12" s="50" t="str">
+        <x:v>Private legal / civil-rights case record</x:v>
+      </x:c>
+      <x:c r="C12" s="50" t="str">
+        <x:v>Strictly private — excluded from public repository</x:v>
+      </x:c>
+      <x:c r="D12" s="50" t="str">
+        <x:v>Not a Zenodo candidate</x:v>
+      </x:c>
+      <x:c r="E12" s="50" t="str">
+        <x:v>Interview statement containing personal, case, housing, and third-party information.</x:v>
+      </x:c>
+      <x:c r="F12" s="50" t="str">
+        <x:v>Preserve unchanged; keep outside public GitHub and marketing; route only through authorized legal/agency channels.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13">
+      <x:c r="A13" s="50" t="str">
+        <x:v>The Summer It Gave Me — Songbook Page</x:v>
+      </x:c>
+      <x:c r="B13" s="50" t="str">
+        <x:v>Original song / music publication</x:v>
+      </x:c>
+      <x:c r="C13" s="50" t="str">
+        <x:v>Public candidate after authorship and rights check</x:v>
+      </x:c>
+      <x:c r="D13" s="50" t="str">
+        <x:v>No match in recovered 60</x:v>
+      </x:c>
+      <x:c r="E13" s="50" t="str">
+        <x:v>Original reflective song page with lyrics, chords, tempo, strumming pattern, and authorship notice.</x:v>
+      </x:c>
+      <x:c r="F13" s="50" t="str">
+        <x:v>Confirm contributions and metadata; create an accessible clean lead sheet; music-rights review before distribution.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="14">
+      <x:c r="A14" s="50" t="str">
+        <x:v>Zenodo(1)</x:v>
+      </x:c>
+      <x:c r="B14" s="50" t="str">
+        <x:v>Duplicate local copy of The Cost of the Foundation</x:v>
+      </x:c>
+      <x:c r="C14" s="50" t="str">
+        <x:v>Duplicate — do not count separately</x:v>
+      </x:c>
+      <x:c r="D14" s="50" t="str">
+        <x:v>Exact local content duplicate</x:v>
+      </x:c>
+      <x:c r="E14" s="50" t="str">
+        <x:v>Duplicate Word copy of The Cost of the Foundation under a generic filename.</x:v>
+      </x:c>
+      <x:c r="F14" s="50" t="str">
+        <x:v>Keep checksum/provenance; designate descriptive filename canonical; exclude from work/publication counts.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="15">
+      <x:c r="A15" s="50" t="str">
+        <x:v>My Evidence Files</x:v>
+      </x:c>
+      <x:c r="B15" s="50" t="str">
+        <x:v>Private legal evidence index / analytical notes</x:v>
+      </x:c>
+      <x:c r="C15" s="50" t="str">
+        <x:v>Strictly private — excluded from public repository</x:v>
+      </x:c>
+      <x:c r="D15" s="50" t="str">
+        <x:v>Not a Zenodo candidate</x:v>
+      </x:c>
+      <x:c r="E15" s="50" t="str">
+        <x:v>Organizational evidence map for a personal legal/civil-rights matter.</x:v>
+      </x:c>
+      <x:c r="F15" s="50" t="str">
+        <x:v>Preserve originals and chain of custody; do not rewrite evidence; share only with authorized recipients.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="16">
+      <x:c r="A16" s="50" t="str">
+        <x:v>Emergency Response Systems Under Institutional Inertia</x:v>
+      </x:c>
+      <x:c r="B16" s="50" t="str">
+        <x:v>Research thesis / public-safety systems design</x:v>
+      </x:c>
+      <x:c r="C16" s="50" t="str">
+        <x:v>Public candidate after evidence and safety review</x:v>
+      </x:c>
+      <x:c r="D16" s="50" t="str">
+        <x:v>No match in recovered 60</x:v>
+      </x:c>
+      <x:c r="E16" s="50" t="str">
+        <x:v>Emergency communications history, dispatcher cognitive load, adoption barriers, and human-led AI dispatch architecture.</x:v>
+      </x:c>
+      <x:c r="F16" s="50" t="str">
+        <x:v>Complete structure and citations; define bounded tasks/failure metrics; public-safety, accessibility, cyber, privacy, labor, legal, and human-factors review.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="17">
+      <x:c r="A17" s="50" t="str">
+        <x:v>The Chicken-Leg Tax</x:v>
+      </x:c>
+      <x:c r="B17" s="50" t="str">
+        <x:v>Social-science essay / research paper</x:v>
+      </x:c>
+      <x:c r="C17" s="50" t="str">
+        <x:v>Public candidate after source and sensitivity review</x:v>
+      </x:c>
+      <x:c r="D17" s="50" t="str">
+        <x:v>No match in recovered 60</x:v>
+      </x:c>
+      <x:c r="E17" s="50" t="str">
+        <x:v>Misogynoir, racial vigilance, emotional safety labor, weathering, and burdens Black women face in ordinary public life.</x:v>
+      </x:c>
+      <x:c r="F17" s="50" t="str">
+        <x:v>Remove conversational scaffolding; verify citations; separate lived experience from general claims; Black-feminist/public-health review.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="18">
+      <x:c r="A18" s="50" t="str">
+        <x:v>Designed to Die</x:v>
+      </x:c>
+      <x:c r="B18" s="50" t="str">
+        <x:v>Systems-exhaustion manifesto / speculative essay</x:v>
+      </x:c>
+      <x:c r="C18" s="50" t="str">
+        <x:v>Editorial development</x:v>
+      </x:c>
+      <x:c r="D18" s="50" t="str">
+        <x:v>No match in recovered 60</x:v>
+      </x:c>
+      <x:c r="E18" s="50" t="str">
+        <x:v>Satirical manifesto on planned obsolescence, housing/income traps, business precarity, subscriptions, ecology, and systems exhaustion.</x:v>
+      </x:c>
+      <x:c r="F18" s="50" t="str">
+        <x:v>Separate memoir, satire, policy claims, and fiction; fact-check; edit for audience; legal and sensitivity review.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="19">
+      <x:c r="A19" s="50" t="str">
+        <x:v>Dragon Café Sanctuary — Phase 1 Baby-Step Deployment Plan</x:v>
+      </x:c>
+      <x:c r="B19" s="50" t="str">
+        <x:v>Business validation and audience-development plan</x:v>
+      </x:c>
+      <x:c r="C19" s="50" t="str">
+        <x:v>Private operating plan; sanitized summary only</x:v>
+      </x:c>
+      <x:c r="D19" s="50" t="str">
+        <x:v>No match in recovered 60</x:v>
+      </x:c>
+      <x:c r="E19" s="50" t="str">
+        <x:v>Low-capital brand, audience, and research sequence before any premises or live-animal operation.</x:v>
+      </x:c>
+      <x:c r="F19" s="50" t="str">
+        <x:v>Check names/handles; research permits, insurance, food, welfare, zoonotic risk, accessibility, and venue rules; demand tests first.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="20">
+      <x:c r="A20" s="50" t="str">
+        <x:v>Professional Reptilian Capture &amp; Control System — Master Product Specification</x:v>
+      </x:c>
+      <x:c r="B20" s="50" t="str">
+        <x:v>Animal-handling product specification / invention</x:v>
+      </x:c>
+      <x:c r="C20" s="50" t="str">
+        <x:v>Private technical development</x:v>
+      </x:c>
+      <x:c r="D20" s="50" t="str">
+        <x:v>No match in recovered 60</x:v>
+      </x:c>
+      <x:c r="E20" s="50" t="str">
+        <x:v>Modular snake-hook and capture-tong specification covering dimensions, materials, ergonomics, safety, and transport.</x:v>
+      </x:c>
+      <x:c r="F20" s="50" t="str">
+        <x:v>Freeze unverified claims; prior-art/standards review; credentialed herpetology, veterinary, welfare, engineering, liability, and field-safety review.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="21">
+      <x:c r="A21" s="50" t="str">
+        <x:v>Dragon Café Sanctuary — Master Business Plan and Immersive Hospitality Blueprint</x:v>
+      </x:c>
+      <x:c r="B21" s="50" t="str">
+        <x:v>Hospitality, education, and animal-sanctuary business plan</x:v>
+      </x:c>
+      <x:c r="C21" s="50" t="str">
+        <x:v>Private business plan; sanitized concept only</x:v>
+      </x:c>
+      <x:c r="D21" s="50" t="str">
+        <x:v>No match in recovered 60</x:v>
+      </x:c>
+      <x:c r="E21" s="50" t="str">
+        <x:v>Luxury reptile lounge combining education, supervised interaction, café service, fantasy hospitality, sanctuary values, and events.</x:v>
+      </x:c>
+      <x:c r="F21" s="50" t="str">
+        <x:v>Jurisdictional feasibility: separation, permits, veterinary oversight, welfare, sanitation, zoonotic risk, insurance, accessibility, staffing, capital, and pilot alternatives.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="22">
+      <x:c r="A22" s="50" t="str">
+        <x:v>Why Superman Ain’t Coming</x:v>
+      </x:c>
+      <x:c r="B22" s="50" t="str">
+        <x:v>Scenario-based sociotechnical governance paper</x:v>
+      </x:c>
+      <x:c r="C22" s="50" t="str">
+        <x:v>Public candidate; IP/source review required</x:v>
+      </x:c>
+      <x:c r="D22" s="50" t="str">
+        <x:v>Supplement states DOI 10.5281/zenodo.18571384 — unverified</x:v>
+      </x:c>
+      <x:c r="E22" s="50" t="str">
+        <x:v>Hypothetical Superman timeline examining emergency management, containment, narrative control, public health, and corporate capture.</x:v>
+      </x:c>
+      <x:c r="F22" s="50" t="str">
+        <x:v>Combine base and supplement; verify DOI/doctrine citations; transformative-use, trademark, quotation, legal, and editorial review.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="23">
+      <x:c r="A23" s="50" t="str">
+        <x:v>Cask &amp; Crunch — Master Legacy Business Plan</x:v>
+      </x:c>
+      <x:c r="B23" s="50" t="str">
+        <x:v>Hospitality / beverage / fermentation business plan</x:v>
+      </x:c>
+      <x:c r="C23" s="50" t="str">
+        <x:v>Private business plan; sanitized summary only</x:v>
+      </x:c>
+      <x:c r="D23" s="50" t="str">
+        <x:v>No match in recovered 60</x:v>
+      </x:c>
+      <x:c r="E23" s="50" t="str">
+        <x:v>Fukuoka launch/expansion plan for specialty beverages, pickle pairing, fermentation, community, and education.</x:v>
+      </x:c>
+      <x:c r="F23" s="50" t="str">
+        <x:v>Japan visa/entity/licensing, food safety, alcohol rules if applicable, localization, demand, capital, unit economics, local legal/accounting review.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="24">
+      <x:c r="A24" s="50" t="str">
+        <x:v>The Pennyworth Papers</x:v>
+      </x:c>
+      <x:c r="B24" s="50" t="str">
+        <x:v>Transformative fan cookbook / character scholarship</x:v>
+      </x:c>
+      <x:c r="C24" s="50" t="str">
+        <x:v>Rights-restricted publication candidate</x:v>
+      </x:c>
+      <x:c r="D24" s="50" t="str">
+        <x:v>No match in recovered 60</x:v>
+      </x:c>
+      <x:c r="E24" s="50" t="str">
+        <x:v>Wayne Manor-inspired culinary reconstruction centered on care, recovery food, household routines, and Alfred Pennyworth.</x:v>
+      </x:c>
+      <x:c r="F24" s="50" t="str">
+        <x:v>Keep full manuscript private; audit canon, quotes, recipes, names, images, credits, trademarks, and commercial fan-work rights.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="25">
+      <x:c r="A25" s="50" t="str">
+        <x:v>Reality Audit Stage 7</x:v>
+      </x:c>
+      <x:c r="B25" s="50" t="str">
+        <x:v>Research milestone / real-data anisotropy analysis</x:v>
+      </x:c>
+      <x:c r="C25" s="50" t="str">
+        <x:v>Public candidate after reproducibility review</x:v>
+      </x:c>
+      <x:c r="D25" s="50" t="str">
+        <x:v>No match in recovered 60</x:v>
+      </x:c>
+      <x:c r="E25" s="50" t="str">
+        <x:v>Move from synthetic validation to public event-data tests for preferred-axis, timing, and clustering anomalies without simulation proof claims.</x:v>
+      </x:c>
+      <x:c r="F25" s="50" t="str">
+        <x:v>Exact dataset/license; preregistration; code/environment/checksums; negative controls; multiple-comparison/selection-bias tests; independent statistics/domain review.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="26">
+      <x:c r="A26" s="50" t="str">
+        <x:v>The Curated Cask — Washington State Business Implementation Plan</x:v>
+      </x:c>
+      <x:c r="B26" s="50" t="str">
+        <x:v>Retail alcohol / cultural experience business plan</x:v>
+      </x:c>
+      <x:c r="C26" s="50" t="str">
+        <x:v>Private business plan; sanitized summary only</x:v>
+      </x:c>
+      <x:c r="D26" s="50" t="str">
+        <x:v>No match in recovered 60</x:v>
+      </x:c>
+      <x:c r="E26" s="50" t="str">
+        <x:v>Small-format premium alcohol retail and guided-tasting concept for the Seattle/Tacoma area.</x:v>
+      </x:c>
+      <x:c r="F26" s="50" t="str">
+        <x:v>Washington licensing, zoning, insurance, age controls, service duties, tasting rules, supplier economics, rent, turns, margin, capital, demand.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="27">
+      <x:c r="A27" s="50" t="str">
+        <x:v>Fukuoka City Startup Visa FAQ capture</x:v>
+      </x:c>
+      <x:c r="B27" s="50" t="str">
+        <x:v>External regulatory reference / source material</x:v>
+      </x:c>
+      <x:c r="C27" s="50" t="str">
+        <x:v>Reference only — do not republish as authored work</x:v>
+      </x:c>
+      <x:c r="D27" s="50" t="str">
+        <x:v>Official-source capture; not a work</x:v>
+      </x:c>
+      <x:c r="E27" s="50" t="str">
+        <x:v>Captured Fukuoka City Startup Visa FAQ and application guidance with source copyright notice.</x:v>
+      </x:c>
+      <x:c r="F27" s="50" t="str">
+        <x:v>Record URL/capture date; current official version and qualified immigration advice; quote narrowly with attribution; do not upload full copy.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="28">
+      <x:c r="A28" s="50" t="str">
+        <x:v>Gotham After Midnight — The Ledger Lies, the City Doesn’t</x:v>
+      </x:c>
+      <x:c r="B28" s="50" t="str">
+        <x:v>Original audio fiction / spoken word using Gotham setting</x:v>
+      </x:c>
+      <x:c r="C28" s="50" t="str">
+        <x:v>Rights-restricted creative work</x:v>
+      </x:c>
+      <x:c r="D28" s="50" t="str">
+        <x:v>No match in recovered 60</x:v>
+      </x:c>
+      <x:c r="E28" s="50" t="str">
+        <x:v>Noir radio monologue on ledgers, delay, bureaucracy, housing pressure, survival, and city memory.</x:v>
+      </x:c>
+      <x:c r="F28" s="50" t="str">
+        <x:v>Separate original commentary from third-party setting/marks; rights/editorial review; develop rights-cleared original-city version.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="29">
+      <x:c r="A29" s="50" t="str">
+        <x:v>Bureaucracy as Physical Violence</x:v>
+      </x:c>
+      <x:c r="B29" s="50" t="str">
+        <x:v>Personal narrative / analytical conversation</x:v>
+      </x:c>
+      <x:c r="C29" s="50" t="str">
+        <x:v>Strictly private source; anonymized essay possible</x:v>
+      </x:c>
+      <x:c r="D29" s="50" t="str">
+        <x:v>No match in recovered 60</x:v>
+      </x:c>
+      <x:c r="E29" s="50" t="str">
+        <x:v>Personal health/housing account followed by an interpretation of bureaucratic violence and historical patterns.</x:v>
+      </x:c>
+      <x:c r="F29" s="50" t="str">
+        <x:v>Protect health/legal/housing details; do not publish raw dialogue; verify claims; legal/medical support as appropriate; separate anonymized essay after review.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="30">
+      <x:c r="A30" s="50" t="str">
+        <x:v>Proto-Theocratic Settler Movements, Social Control, and the Myth of Religious Freedom in Early Colonial America</x:v>
+      </x:c>
+      <x:c r="B30" s="50" t="str">
+        <x:v>Historical sociology / political theology paper</x:v>
+      </x:c>
+      <x:c r="C30" s="50" t="str">
+        <x:v>Public candidate after scholarly review</x:v>
+      </x:c>
+      <x:c r="D30" s="50" t="str">
+        <x:v>No match in recovered 60</x:v>
+      </x:c>
+      <x:c r="E30" s="50" t="str">
+        <x:v>Analysis of Puritan governance, high-control religious structures, settler colonialism, dissent suppression, and religious freedom limits.</x:v>
+      </x:c>
+      <x:c r="F30" s="50" t="str">
+        <x:v>Verify citations/quotes; refine terminology; historians of religion, Indigenous history, colonial studies, and sensitivity review.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="31">
+      <x:c r="A31" s="50" t="str">
+        <x:v>Why Superman Ain’t Coming: Additional</x:v>
+      </x:c>
+      <x:c r="B31" s="50" t="str">
+        <x:v>Supplement — not a separate work count</x:v>
+      </x:c>
+      <x:c r="C31" s="50" t="str">
+        <x:v>Version component of public candidate</x:v>
+      </x:c>
+      <x:c r="D31" s="50" t="str">
+        <x:v>States DOI 10.5281/zenodo.18571384 — unverified</x:v>
+      </x:c>
+      <x:c r="E31" s="50" t="str">
+        <x:v>Supplement covering media narratives, corporate capture, liability, insurance, monetization, and intellectual property.</x:v>
+      </x:c>
+      <x:c r="F31" s="50" t="str">
+        <x:v>Merge/cross-reference as supplement; verify DOI live; preserve lineage; avoid double-counting.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="32">
+      <x:c r="A32" s="50" t="str">
+        <x:v>Edge Cases, High Signal, and Institutional Containment — Full Course Syllabus</x:v>
+      </x:c>
+      <x:c r="B32" s="50" t="str">
+        <x:v>Curriculum package / systems course</x:v>
+      </x:c>
+      <x:c r="C32" s="50" t="str">
+        <x:v>Public candidate after source, safety, and pedagogy review</x:v>
+      </x:c>
+      <x:c r="D32" s="50" t="str">
+        <x:v>No match in recovered 60</x:v>
+      </x:c>
+      <x:c r="E32" s="50" t="str">
+        <x:v>Ten-week diagnostic/navigation course combining institutional analysis, edge-case theory, documentation strategy, survival tools, and advocate training.</x:v>
+      </x:c>
+      <x:c r="F32" s="50" t="str">
+        <x:v>Bound assertions; cited readings; learner safeguards; accessibility; rubrics; legal/trauma-aware review; supervised pilot.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="33">
+      <x:c r="A33" s="50" t="str">
+        <x:v>The Systems Survival Playbook — Field Guide</x:v>
+      </x:c>
+      <x:c r="B33" s="50" t="str">
+        <x:v>Course companion / field guide</x:v>
+      </x:c>
+      <x:c r="C33" s="50" t="str">
+        <x:v>Curriculum component — not separate work</x:v>
+      </x:c>
+      <x:c r="D33" s="50" t="str">
+        <x:v>No match in recovered 60</x:v>
+      </x:c>
+      <x:c r="E33" s="50" t="str">
+        <x:v>Compact guide on documentation, dialogue, silence, helpers, and exit within difficult institutions.</x:v>
+      </x:c>
+      <x:c r="F33" s="50" t="str">
+        <x:v>Bound categorical claims; add emergency/legal/disability/referral guidance; test with tenants, caseworkers, and legal reviewers.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="34">
+      <x:c r="A34" s="50" t="str">
+        <x:v>How to Stay Legible Without Becoming a Target — Map</x:v>
+      </x:c>
+      <x:c r="B34" s="50" t="str">
+        <x:v>Course companion / communication map</x:v>
+      </x:c>
+      <x:c r="C34" s="50" t="str">
+        <x:v>Curriculum component — not separate work</x:v>
+      </x:c>
+      <x:c r="D34" s="50" t="str">
+        <x:v>No match in recovered 60</x:v>
+      </x:c>
+      <x:c r="E34" s="50" t="str">
+        <x:v>Legibility-level model and green/yellow/red filter for institutional communication.</x:v>
+      </x:c>
+      <x:c r="F34" s="50" t="str">
+        <x:v>Validate model; add context, exceptions, legal-record duties, escalation routes, and warnings against withholding material facts.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="35">
+      <x:c r="A35" s="50" t="str">
+        <x:v>The Systems Survival Handbook</x:v>
+      </x:c>
+      <x:c r="B35" s="50" t="str">
+        <x:v>Public-facing handbook / curriculum component</x:v>
+      </x:c>
+      <x:c r="C35" s="50" t="str">
+        <x:v>Canonical handbook candidate</x:v>
+      </x:c>
+      <x:c r="D35" s="50" t="str">
+        <x:v>No match in recovered 60</x:v>
+      </x:c>
+      <x:c r="E35" s="50" t="str">
+        <x:v>Trauma-aware handbook for tenants, caregivers, advocates, and caseworkers with survival rules and advocate training.</x:v>
+      </x:c>
+      <x:c r="F35" s="50" t="str">
+        <x:v>Canonicalize; merge guide/map appendices; source claims; jurisdiction/crisis disclaimers; accessibility/legal/usability review.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="36">
+      <x:c r="A36" s="50" t="str">
+        <x:v>Edge Cases with High Signal</x:v>
+      </x:c>
+      <x:c r="B36" s="50" t="str">
+        <x:v>Research paper / parent theory</x:v>
+      </x:c>
+      <x:c r="C36" s="50" t="str">
+        <x:v>Public candidate after evidence/editorial review</x:v>
+      </x:c>
+      <x:c r="D36" s="50" t="str">
+        <x:v>Two local versions; one work lineage</x:v>
+      </x:c>
+      <x:c r="E36" s="50" t="str">
+        <x:v>Theory of containment, catch-and-kill dynamics, procedural harm, and institutional self-preservation around coherent edge cases.</x:v>
+      </x:c>
+      <x:c r="F36" s="50" t="str">
+        <x:v>Select canonical version; preserve lineage; verify citations/case claims; distinguish hypotheses; independent systems/legal/public-administration review.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="37">
+      <x:c r="A37" s="50" t="str">
+        <x:v>Are you a Edge Cases with High Signal</x:v>
+      </x:c>
+      <x:c r="B37" s="50" t="str">
+        <x:v>Alternate draft</x:v>
+      </x:c>
+      <x:c r="C37" s="50" t="str">
+        <x:v>Duplicate lineage — not separate work</x:v>
+      </x:c>
+      <x:c r="D37" s="50" t="str">
+        <x:v>Same paper family</x:v>
+      </x:c>
+      <x:c r="E37" s="50" t="str">
+        <x:v>Alternate Edge Cases draft with housing case-study and political-economy framing.</x:v>
+      </x:c>
+      <x:c r="F37" s="50" t="str">
+        <x:v>Diff against canonical; protect personal case appendix; retain unique theory with provenance; no raw identifying facts.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="38">
+      <x:c r="A38" s="50" t="str">
+        <x:v>Interpretive Helpers and the Moral Architecture of Institutional Harm</x:v>
+      </x:c>
+      <x:c r="B38" s="50" t="str">
+        <x:v>Research paper plus private case addenda</x:v>
+      </x:c>
+      <x:c r="C38" s="50" t="str">
+        <x:v>Private until case material separated</x:v>
+      </x:c>
+      <x:c r="D38" s="50" t="str">
+        <x:v>No match in recovered 60</x:v>
+      </x:c>
+      <x:c r="E38" s="50" t="str">
+        <x:v>Taxonomy of institutional helpers, ethical orientations, credibility asymmetry, and harm, plus case-specific exhibits.</x:v>
+      </x:c>
+      <x:c r="F38" s="50" t="str">
+        <x:v>Split general paper from personal/legal evidence; audit citations/claims; ethics, legal, critical-race, and public-administration review.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="39">
+      <x:c r="A39" s="50" t="str">
+        <x:v>thing.docx</x:v>
+      </x:c>
+      <x:c r="B39" s="50" t="str">
+        <x:v>Empty placeholder</x:v>
+      </x:c>
+      <x:c r="C39" s="50" t="str">
+        <x:v>No publication value</x:v>
+      </x:c>
+      <x:c r="D39" s="50" t="str">
+        <x:v>Empty file; not a work</x:v>
+      </x:c>
+      <x:c r="E39" s="50" t="str">
+        <x:v>Empty Word document.</x:v>
+      </x:c>
+      <x:c r="F39" s="50" t="str">
+        <x:v>Do not count; retain checksum only if provenance matters, otherwise archive outside active portfolio.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="40">
+      <x:c r="A40" s="50" t="str">
+        <x:v>Cross-Reference Map — Commons Socio-Technical Poverty Corpus</x:v>
+      </x:c>
+      <x:c r="B40" s="50" t="str">
+        <x:v>Portfolio architecture / corpus map</x:v>
+      </x:c>
+      <x:c r="C40" s="50" t="str">
+        <x:v>Private working index; sanitized version possible</x:v>
+      </x:c>
+      <x:c r="D40" s="50" t="str">
+        <x:v>Support artifact</x:v>
+      </x:c>
+      <x:c r="E40" s="50" t="str">
+        <x:v>Dependency map across diagnosis, mechanisms, credibility, coercion, outcomes, and case evidence.</x:v>
+      </x:c>
+      <x:c r="F40" s="50" t="str">
+        <x:v>Map canonical filenames, versions, evidence levels, public/private status, citations, dependencies, and missing artifacts; sanitize case details.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="41">
+      <x:c r="A41" s="50" t="str">
+        <x:v>Butterflies and Weapons</x:v>
+      </x:c>
+      <x:c r="B41" s="50" t="str">
+        <x:v>Long-form systems manuscript / manifesto</x:v>
+      </x:c>
+      <x:c r="C41" s="50" t="str">
+        <x:v>Public candidate after substantial review</x:v>
+      </x:c>
+      <x:c r="D41" s="50" t="str">
+        <x:v>No match in recovered 60</x:v>
+      </x:c>
+      <x:c r="E41" s="50" t="str">
+        <x:v>Book contrasting individual empathy with collective violence, domination, civilizational adolescence, and moral stagnation.</x:v>
+      </x:c>
+      <x:c r="F41" s="50" t="str">
+        <x:v>Bound and source claims; separate metaphor/evidence/lived experience/manifesto; multidisciplinary scholarly, sensitivity, and editorial review.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="42">
+      <x:c r="A42" s="50" t="str">
+        <x:v>Butterflies and Weapons — Expanded Manuscript</x:v>
+      </x:c>
+      <x:c r="B42" s="50" t="str">
+        <x:v>Expanded version of existing work</x:v>
+      </x:c>
+      <x:c r="C42" s="50" t="str">
+        <x:v>Canonical-version candidate; not separate work</x:v>
+      </x:c>
+      <x:c r="D42" s="50" t="str">
+        <x:v>Expanded local version</x:v>
+      </x:c>
+      <x:c r="E42" s="50" t="str">
+        <x:v>Expanded manuscript across civilizational maturity, domination, systems theory, casebook, intellectual biography, and nonviolent reflection.</x:v>
+      </x:c>
+      <x:c r="F42" s="50" t="str">
+        <x:v>Diff versions; designate canonical; source ledger; remove duplication/conversational residue; multidisciplinary review/edit.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="43">
+      <x:c r="A43" s="50" t="str">
+        <x:v>Coercion Through Procedure as Poverty Infrastructure</x:v>
+      </x:c>
+      <x:c r="B43" s="50" t="str">
+        <x:v>Case-study paper using protected housing evidence</x:v>
+      </x:c>
+      <x:c r="C43" s="50" t="str">
+        <x:v>Strictly private pending legal/de-identification review</x:v>
+      </x:c>
+      <x:c r="D43" s="50" t="str">
+        <x:v>No match in recovered 60</x:v>
+      </x:c>
+      <x:c r="E43" s="50" t="str">
+        <x:v>Housing timeline linked to procedural coercion, debt re-aging, retaliatory sequencing, maternal triage, and poverty infrastructure.</x:v>
+      </x:c>
+      <x:c r="F43" s="50" t="str">
+        <x:v>Keep evidence private; counsel verifies privilege/accuracy/retaliation/public-record risk; formal de-identification; methods/housing-law/ethics review.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="44">
+      <x:c r="A44" s="50" t="str">
+        <x:v>The Pointlessness for the Target, the Security for Everyone Else</x:v>
+      </x:c>
+      <x:c r="B44" s="50" t="str">
+        <x:v>Socio-technical systems research paper</x:v>
+      </x:c>
+      <x:c r="C44" s="50" t="str">
+        <x:v>Public candidate after evidence/legal review</x:v>
+      </x:c>
+      <x:c r="D44" s="50" t="str">
+        <x:v>No match in recovered 60</x:v>
+      </x:c>
+      <x:c r="E44" s="50" t="str">
+        <x:v>Futile reporting, risk displacement, institutional self-preservation, procedural reassurance, and unequal consequences.</x:v>
+      </x:c>
+      <x:c r="F44" s="50" t="str">
+        <x:v>Verify regulations/data/citations; calibrate design claims; separate general theory from case inference; multidisciplinary review.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="45">
+      <x:c r="A45" s="50" t="str">
+        <x:v>Self-Generated Harm</x:v>
+      </x:c>
+      <x:c r="B45" s="50" t="str">
+        <x:v>Structural impact paper</x:v>
+      </x:c>
+      <x:c r="C45" s="50" t="str">
+        <x:v>Public candidate after evidence/scholarly review</x:v>
+      </x:c>
+      <x:c r="D45" s="50" t="str">
+        <x:v>No match in recovered 60</x:v>
+      </x:c>
+      <x:c r="E45" s="50" t="str">
+        <x:v>System incentives, engineered scarcity, proceduralized cruelty, exhaustion, denial, and suppressed feedback.</x:v>
+      </x:c>
+      <x:c r="F45" s="50" t="str">
+        <x:v>Operationalize scope; source claims; distinguish design/incentive/outcome; add counterexamples/falsification; systems/economics/history/policy review.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="46">
+      <x:c r="A46" s="50" t="str">
+        <x:v>Credibility Asymmetry and Risk-Avoidance in Socio-Technical Housing Systems</x:v>
+      </x:c>
+      <x:c r="B46" s="50" t="str">
+        <x:v>Case-linked research paper</x:v>
+      </x:c>
+      <x:c r="C46" s="50" t="str">
+        <x:v>Strictly private pending documentary/legal review</x:v>
+      </x:c>
+      <x:c r="D46" s="50" t="str">
+        <x:v>No match in recovered 60</x:v>
+      </x:c>
+      <x:c r="E46" s="50" t="str">
+        <x:v>Unequal tolerance for AI-assisted synthesis, racialized credibility, risk avoidance, and tenant communication restrictions.</x:v>
+      </x:c>
+      <x:c r="F46" s="50" t="str">
+        <x:v>Preserve correspondence; verify quotes/chronology; counsel review names/allegations; anonymize theory; no identifying evidence publication.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="47">
+      <x:c r="A47" s="50" t="str">
+        <x:v>Legibility, Risk Avoidance, and the Procedural Suppression of Racialized Credibility</x:v>
+      </x:c>
+      <x:c r="B47" s="50" t="str">
+        <x:v>Socio-technical systems research paper</x:v>
+      </x:c>
+      <x:c r="C47" s="50" t="str">
+        <x:v>Public candidate after evidence/sensitivity review</x:v>
+      </x:c>
+      <x:c r="D47" s="50" t="str">
+        <x:v>No match in recovered 60</x:v>
+      </x:c>
+      <x:c r="E47" s="50" t="str">
+        <x:v>Translation denial, institutional legibility, ambiguity, AI articulation, and the racialized credibility double bind.</x:v>
+      </x:c>
+      <x:c r="F47" s="50" t="str">
+        <x:v>Validate mechanism or label conceptual; citations, counter-hypotheses, limitations; ethics/critical-race/AI/access/legal review.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="48">
+      <x:c r="A48" s="50" t="str">
+        <x:v>Procedural Harm and the Architecture of Disappearing Responsibility</x:v>
+      </x:c>
+      <x:c r="B48" s="50" t="str">
+        <x:v>Structural reflection / essay</x:v>
+      </x:c>
+      <x:c r="C48" s="50" t="str">
+        <x:v>Public candidate after evidence/editorial review</x:v>
+      </x:c>
+      <x:c r="D48" s="50" t="str">
+        <x:v>No match in recovered 60</x:v>
+      </x:c>
+      <x:c r="E48" s="50" t="str">
+        <x:v>Proceduralized harm, diffusion of responsibility, controlled comfort, defensive ambiguity, and linguistic control.</x:v>
+      </x:c>
+      <x:c r="F48" s="50" t="str">
+        <x:v>Choose genre; source claims; add limitations; legal, historical, critical-race, and editorial review.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="49">
+      <x:c r="A49" s="50" t="str">
+        <x:v>When Housing Debt Consumes the Body</x:v>
+      </x:c>
+      <x:c r="B49" s="50" t="str">
+        <x:v>Public-health and housing-systems paper</x:v>
+      </x:c>
+      <x:c r="C49" s="50" t="str">
+        <x:v>Private until health/personal material separated</x:v>
+      </x:c>
+      <x:c r="D49" s="50" t="str">
+        <x:v>Two duplicate local filenames</x:v>
+      </x:c>
+      <x:c r="E49" s="50" t="str">
+        <x:v>Housing arrears connected to stress physiology, workability, parenting burden, health degradation, mortality, and funeral insecurity.</x:v>
+      </x:c>
+      <x:c r="F49" s="50" t="str">
+        <x:v>Canonicalize; remove private ending; verify medical/mortality claims; no individual diagnosis; epidemiology/housing-health/clinical/legal/ethics review.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="50">
+      <x:c r="A50" s="50" t="str">
+        <x:v>Human Outcomes, Workability, and Mortality in Public Housing Arrears Systems</x:v>
+      </x:c>
+      <x:c r="B50" s="50" t="str">
+        <x:v>Duplicate local copy / alternate filename</x:v>
+      </x:c>
+      <x:c r="C50" s="50" t="str">
+        <x:v>Duplicate lineage — not separate work</x:v>
+      </x:c>
+      <x:c r="D50" s="50" t="str">
+        <x:v>Duplicates When Housing Debt Consumes the Body</x:v>
+      </x:c>
+      <x:c r="E50" s="50" t="str">
+        <x:v>Alternate filename for the same housing-debt/health manuscript.</x:v>
+      </x:c>
+      <x:c r="F50" s="50" t="str">
+        <x:v>Retain checksum/provenance; consolidate under canonical title; exclude from counts.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="51">
+      <x:c r="A51" s="50" t="str">
+        <x:v>The Re-Aging Debt Trap in Public Housing Enforcement Systems</x:v>
+      </x:c>
+      <x:c r="B51" s="50" t="str">
+        <x:v>Case-linked housing-debt paper</x:v>
+      </x:c>
+      <x:c r="C51" s="50" t="str">
+        <x:v>Strictly private pending ledger/legal/de-identification review</x:v>
+      </x:c>
+      <x:c r="D51" s="50" t="str">
+        <x:v>Filename differs from manuscript title</x:v>
+      </x:c>
+      <x:c r="E51" s="50" t="str">
+        <x:v>Arrears reinstatement, repayment default triggers, payment allocation, ledger opacity, exhaustion, and perpetual indebtedness.</x:v>
+      </x:c>
+      <x:c r="F51" s="50" t="str">
+        <x:v>Verify mechanisms against agreements/ledgers/rules/law/accounting; separate case from prevalence; counsel/accountant/methods/tenant review.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="52">
+      <x:c r="A52" s="50" t="str">
+        <x:v>When the Ledger Breaks — Socio-Technical Accountability Case Study and Training Module</x:v>
+      </x:c>
+      <x:c r="B52" s="50" t="str">
+        <x:v>Housing-ledger case study, policy memo, training, and judicial-brief family</x:v>
+      </x:c>
+      <x:c r="C52" s="50" t="str">
+        <x:v>Strictly private pending legal/de-identification/evidence review</x:v>
+      </x:c>
+      <x:c r="D52" s="50" t="str">
+        <x:v>Three components: training module, case study, and named exhibit packet</x:v>
+      </x:c>
+      <x:c r="E52" s="50" t="str">
+        <x:v>Integrated case and training family on public-housing ledger continuity, certified reconciliation, accountability, and rapid detection of ledger failures.</x:v>
+      </x:c>
+      <x:c r="F52" s="50" t="str">
+        <x:v>Keep identifying evidence private; preserve originals; housing counsel/accounting review; separately de-identified teaching edition only with consent and ethics review.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="53">
+      <x:c r="A53" s="50" t="str">
+        <x:v>Mya Brown Exhibit Packet — Ledger Continuity Break and Demand for Certified Reconciliation</x:v>
+      </x:c>
+      <x:c r="B53" s="50" t="str">
+        <x:v>Protected legal evidence packet</x:v>
+      </x:c>
+      <x:c r="C53" s="50" t="str">
+        <x:v>Strictly private legal evidence; not a publication work</x:v>
+      </x:c>
+      <x:c r="D53" s="50" t="str">
+        <x:v>Support component — not separate work</x:v>
+      </x:c>
+      <x:c r="E53" s="50" t="str">
+        <x:v>Case-specific identifying housing, ledger, balance, personnel, chronology, and settlement material.</x:v>
+      </x:c>
+      <x:c r="F53" s="50" t="str">
+        <x:v>Never place on public GitHub; preserve chain of custody/hash; restrict access; counsel controls disclosure, redaction, and derivative use.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="54">
+      <x:c r="A54" s="50" t="str">
+        <x:v>GPT chat true personality.docx</x:v>
+      </x:c>
+      <x:c r="B54" s="50" t="str">
+        <x:v>Empty placeholder</x:v>
+      </x:c>
+      <x:c r="C54" s="50" t="str">
+        <x:v>No publication value</x:v>
+      </x:c>
+      <x:c r="D54" s="50" t="str">
+        <x:v>Empty file; not a work</x:v>
+      </x:c>
+      <x:c r="E54" s="50" t="str">
+        <x:v>Empty Word document.</x:v>
+      </x:c>
+      <x:c r="F54" s="50" t="str">
+        <x:v>Do not count; retain checksum only if provenance matters, otherwise archive outside active portfolio.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="55">
+      <x:c r="A55" s="50" t="str">
+        <x:v>Black Women as a Threatened Population</x:v>
+      </x:c>
+      <x:c r="B55" s="50" t="str">
+        <x:v>Public-health, social-science, and Black feminist research paper</x:v>
+      </x:c>
+      <x:c r="C55" s="50" t="str">
+        <x:v>Public candidate only after rigorous evidence/sensitivity review</x:v>
+      </x:c>
+      <x:c r="D55" s="50" t="str">
+        <x:v>No match in recovered 60</x:v>
+      </x:c>
+      <x:c r="E55" s="50" t="str">
+        <x:v>Structural threats to Black women through health, violence, institutional, demographic, and historical lenses, plus a psychological companion essay.</x:v>
+      </x:c>
+      <x:c r="F55" s="50" t="str">
+        <x:v>Define metaphor/scope; verify every table/statistic with primary sources; remove residue; Black feminist/public-health/legal/statistical/community review.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="56">
+      <x:c r="A56" s="50" t="str">
+        <x:v>The Black Women’s Truth Ledger</x:v>
+      </x:c>
+      <x:c r="B56" s="50" t="str">
+        <x:v>Documentation, evidence, and accountability framework</x:v>
+      </x:c>
+      <x:c r="C56" s="50" t="str">
+        <x:v>Public framework candidate after ethics/privacy review</x:v>
+      </x:c>
+      <x:c r="D56" s="50" t="str">
+        <x:v>No match in recovered 60</x:v>
+      </x:c>
+      <x:c r="E56" s="50" t="str">
+        <x:v>Tiered-claims and receipts architecture for documenting harms, mechanisms, interventions, and technology constraints affecting Black women.</x:v>
+      </x:c>
+      <x:c r="F56" s="50" t="str">
+        <x:v>Remove chat residue; specify governance, consent, minimization, correction, access, retention, de-identification, and community oversight; privacy-safe pilot.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="57">
+      <x:c r="A57" s="50" t="str">
+        <x:v>A Grounded Conversation on Maturity, Collapse, and the Possibility of Adulthood</x:v>
+      </x:c>
+      <x:c r="B57" s="50" t="str">
+        <x:v>Dialogue appendix / support artifact</x:v>
+      </x:c>
+      <x:c r="C57" s="50" t="str">
+        <x:v>Private working appendix; edited excerpt possible</x:v>
+      </x:c>
+      <x:c r="D57" s="50" t="str">
+        <x:v>Civilizational-maturity support — not separate work</x:v>
+      </x:c>
+      <x:c r="E57" s="50" t="str">
+        <x:v>Dialogue on maturity, collapse, structural irreversibility, and adult civilizational responsibility.</x:v>
+      </x:c>
+      <x:c r="F57" s="50" t="str">
+        <x:v>Use as appendix; remove personal dialogue and unsupported assertions; publish only rights-cleared, sourced analysis.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="58">
+      <x:c r="A58" s="50" t="str">
+        <x:v>What Would It Take to Break the Historical Pattern</x:v>
+      </x:c>
+      <x:c r="B58" s="50" t="str">
+        <x:v>Historical systems and civilizational-maturity addendum</x:v>
+      </x:c>
+      <x:c r="C58" s="50" t="str">
+        <x:v>Public candidate after source/rights review</x:v>
+      </x:c>
+      <x:c r="D58" s="50" t="str">
+        <x:v>Addendum E</x:v>
+      </x:c>
+      <x:c r="E58" s="50" t="str">
+        <x:v>Guardrails, anti-reconsolidation, and shared reality as conditions for interrupting recurrent historical failure.</x:v>
+      </x:c>
+      <x:c r="F58" s="50" t="str">
+        <x:v>Verify examples; define mechanisms/falsification; separate analogy from evidence; rights review fictional references; history/governance/editorial review.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="59">
+      <x:c r="A59" s="50" t="str">
+        <x:v>I Am What I Am — Career Translation</x:v>
+      </x:c>
+      <x:c r="B59" s="50" t="str">
+        <x:v>Career-development and portfolio translation</x:v>
+      </x:c>
+      <x:c r="C59" s="50" t="str">
+        <x:v>Private career source; sanitized derivative possible</x:v>
+      </x:c>
+      <x:c r="D59" s="50" t="str">
+        <x:v>No match in recovered 60</x:v>
+      </x:c>
+      <x:c r="E59" s="50" t="str">
+        <x:v>Translation of socio-technical accountability work into training, curriculum, research, and systems-design roles.</x:v>
+      </x:c>
+      <x:c r="F59" s="50" t="str">
+        <x:v>Keep planning private; verify role/credential claims; create separate sanitized resume, portfolio summary, and role-target matrix.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="60">
+      <x:c r="A60" s="51" t="str">
+        <x:v>A Longitudinal Analysis of Human Reform, Regression, and Relapse</x:v>
+      </x:c>
+      <x:c r="B60" s="51" t="str">
+        <x:v>Historical systems-analysis addendum</x:v>
+      </x:c>
+      <x:c r="C60" s="51" t="str">
+        <x:v>Public candidate after rigorous historical review</x:v>
+      </x:c>
+      <x:c r="D60" s="51" t="str">
+        <x:v>Addendum D</x:v>
+      </x:c>
+      <x:c r="E60" s="51" t="str">
+        <x:v>Historical cycle and learning-retention scale for reform, regression, relapse, and institutional memory.</x:v>
+      </x:c>
+      <x:c r="F60" s="51" t="str">
+        <x:v>Operationalize scale; predefine cases/coding; test counterexamples; calibrate claims; sources and history/comparative-politics/methods review.</x:v>
+      </x:c>
+    </x:row>
+  </x:sheetData>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <x:tableParts count="1">
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0688e04038b64e6a"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
docs: classify intake batch 7 by commercial and mission lanes
Record 69 source files representing 49 unique works and add market routes and Civic Continuum roles while preserving privacy, rights, evidence, and safety boundaries.
</commit_message>
<xml_diff>
--- a/docs/portfolio/zenodo/Mya_Brown_Zenodo_Master_Catalog_and_Development_Pipeline.xlsx
+++ b/docs/portfolio/zenodo/Mya_Brown_Zenodo_Master_Catalog_and_Development_Pipeline.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="R9c507850fd004a40"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Master Catalog" sheetId="2" r:id="R8beffc184cd14c5f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Development Pipeline" sheetId="3" r:id="R5b87a5335f7749ed"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Validation &amp; Partners" sheetId="4" r:id="Rc61dd578c0bd4ee2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="5" r:id="R64c0758339004c8e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Document Intake" sheetId="6" r:id="R11830168a2bb4fa7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="R320d3ad58e984d3a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Master Catalog" sheetId="2" r:id="R523819f4e9204128"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Development Pipeline" sheetId="3" r:id="R44cf690faae647a7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Validation &amp; Partners" sheetId="4" r:id="R4ef9983d5da74a1a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="5" r:id="R6aced7bee5364136"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Document Intake" sheetId="6" r:id="Rc80079e7361d489f"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -365,14 +365,16 @@
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="DocumentIntake" displayName="DocumentIntake" ref="A1:F60" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:tableColumns count="6">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="DocumentIntake" displayName="DocumentIntake" ref="A1:H70" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:tableColumns count="8">
     <x:tableColumn id="1" name="Source document"/>
     <x:tableColumn id="2" name="Portfolio type"/>
     <x:tableColumn id="3" name="Release disposition"/>
     <x:tableColumn id="4" name="Zenodo match status"/>
     <x:tableColumn id="5" name="Working description"/>
     <x:tableColumn id="6" name="Next evidence gate"/>
+    <x:tableColumn id="7" name="Commercial route"/>
+    <x:tableColumn id="8" name="Civic Continuum role"/>
   </x:tableColumns>
   <x:tableStyleInfo name="TableStyleMedium4" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </x:table>
@@ -651,7 +653,7 @@
         <x:v>Local source files / unique works</x:v>
       </x:c>
       <x:c r="B6" s="24" t="str">
-        <x:v>59 files / 45 unique</x:v>
+        <x:v>69 files / 49 unique</x:v>
       </x:c>
       <x:c r="C6" s="52"/>
       <x:c r="D6" s="52"/>
@@ -3336,7 +3338,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf59d0a835c92418f"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R54d2d4a5b8274148"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4667,7 +4669,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R07b416a7f00148a3"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9faa5065dc6344ce"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4926,7 +4928,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra5ed2f2eba674c70"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R39a11e7f64454d1e"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5118,7 +5120,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf9b28abd347a4872"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra483bf9210eb4886"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5134,8 +5136,10 @@
     <x:col min="2" max="2" width="34" hidden="0" customWidth="1"/>
     <x:col min="3" max="3" width="34" hidden="0" customWidth="1"/>
     <x:col min="4" max="4" width="28" hidden="0" customWidth="1"/>
-    <x:col min="5" max="5" width="70" hidden="0" customWidth="1"/>
-    <x:col min="6" max="6" width="76" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="64" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="70" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="66" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="66" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1">
@@ -5157,6 +5161,12 @@
       <x:c r="F1" s="49" t="str">
         <x:v>Next evidence gate</x:v>
       </x:c>
+      <x:c r="G1" s="49" t="str">
+        <x:v>Commercial route</x:v>
+      </x:c>
+      <x:c r="H1" s="49" t="str">
+        <x:v>Civic Continuum role</x:v>
+      </x:c>
     </x:row>
     <x:row r="2">
       <x:c r="A2" s="50" t="str">
@@ -5177,6 +5187,12 @@
       <x:c r="F2" s="50" t="str">
         <x:v>Normalize citations and claims; attach CERL; final PDF; independent subject-matter and legal review.</x:v>
       </x:c>
+      <x:c r="G2" s="50" t="str">
+        <x:v>Sourced paper or brief, then paid talks, workshops, consulting, licensing, or a reader-facing book after review.</x:v>
+      </x:c>
+      <x:c r="H2" s="50" t="str">
+        <x:v>Public framework: builds the case for durable guardrails, shared reality, institutional memory, and stable self-governance.</x:v>
+      </x:c>
     </x:row>
     <x:row r="3">
       <x:c r="A3" s="50" t="str">
@@ -5197,6 +5213,12 @@
       <x:c r="F3" s="50" t="str">
         <x:v>Repair citation artifacts; verify implementation claims; add evidence labels; independent security/governance review.</x:v>
       </x:c>
+      <x:c r="G3" s="50" t="str">
+        <x:v>Bounded demonstrator, paid pilot, subscription, or enterprise license after tests, consent controls, security review, and support.</x:v>
+      </x:c>
+      <x:c r="H3" s="50" t="str">
+        <x:v>Physical proof: turns claims into measured prototypes, independent review, production evidence, and useful products.</x:v>
+      </x:c>
     </x:row>
     <x:row r="4">
       <x:c r="A4" s="50" t="str">
@@ -5217,6 +5239,12 @@
       <x:c r="F4" s="50" t="str">
         <x:v>Audit every factual claim and citation; separate evidence from inference; add safeguard counter-cases; external review.</x:v>
       </x:c>
+      <x:c r="G4" s="50" t="str">
+        <x:v>Sourced paper or brief, then paid talks, workshops, consulting, licensing, or a reader-facing book after review.</x:v>
+      </x:c>
+      <x:c r="H4" s="50" t="str">
+        <x:v>Portfolio support: preserves provenance, strengthens evidence, or supports delivery without overstating readiness.</x:v>
+      </x:c>
     </x:row>
     <x:row r="5">
       <x:c r="A5" s="50" t="str">
@@ -5237,6 +5265,12 @@
       <x:c r="F5" s="50" t="str">
         <x:v>Use as canonical candidate; reconcile citations, version and license; remove conversational residue; technical/legal/editorial review.</x:v>
       </x:c>
+      <x:c r="G5" s="50" t="str">
+        <x:v>Rights-cleared print, ebook, audiobook, music, or serialized edition after professional editing and launch preparation.</x:v>
+      </x:c>
+      <x:c r="H5" s="50" t="str">
+        <x:v>Accountability practice: converts system failures into auditable methods, training, paid services, and institutional repair tools.</x:v>
+      </x:c>
     </x:row>
     <x:row r="6">
       <x:c r="A6" s="50" t="str">
@@ -5257,6 +5291,12 @@
       <x:c r="F6" s="50" t="str">
         <x:v>Diff against refined Blue Book; preserve unique material in version history; do not release as independent work without lineage note.</x:v>
       </x:c>
+      <x:c r="G6" s="50" t="str">
+        <x:v>Rights-cleared print, ebook, audiobook, music, or serialized edition after professional editing and launch preparation.</x:v>
+      </x:c>
+      <x:c r="H6" s="50" t="str">
+        <x:v>Accountability practice: converts system failures into auditable methods, training, paid services, and institutional repair tools.</x:v>
+      </x:c>
     </x:row>
     <x:row r="7">
       <x:c r="A7" s="50" t="str">
@@ -5277,6 +5317,12 @@
       <x:c r="F7" s="50" t="str">
         <x:v>Keep design details private; complete corrected-system baseline and calibrated measurements; independent brake/test-safety review.</x:v>
       </x:c>
+      <x:c r="G7" s="50" t="str">
+        <x:v>Prior art → requirements → simulation/bench proof → safety review → prototype → pilot → manufacturing → truthful launch.</x:v>
+      </x:c>
+      <x:c r="H7" s="50" t="str">
+        <x:v>Physical proof: turns claims into measured prototypes, independent review, production evidence, and useful products.</x:v>
+      </x:c>
     </x:row>
     <x:row r="8">
       <x:c r="A8" s="50" t="str">
@@ -5297,6 +5343,12 @@
       <x:c r="F8" s="50" t="str">
         <x:v>Verify specifications; add chassis/market caveats; trademark, safety, rights, and editorial review.</x:v>
       </x:c>
+      <x:c r="G8" s="50" t="str">
+        <x:v>Rights-cleared print, ebook, audiobook, music, or serialized edition after professional editing and launch preparation.</x:v>
+      </x:c>
+      <x:c r="H8" s="50" t="str">
+        <x:v>Physical proof: turns claims into measured prototypes, independent review, production evidence, and useful products.</x:v>
+      </x:c>
     </x:row>
     <x:row r="9">
       <x:c r="A9" s="50" t="str">
@@ -5317,6 +5369,12 @@
       <x:c r="F9" s="50" t="str">
         <x:v>Do not present as official; separate original pedagogy from third-party IP or create a rights-cleared original academy.</x:v>
       </x:c>
+      <x:c r="G9" s="50" t="str">
+        <x:v>Rights-cleared workbook, facilitator kit, cohort course, institutional license, or consulting package after review and pilot evidence.</x:v>
+      </x:c>
+      <x:c r="H9" s="50" t="str">
+        <x:v>Audience and revenue: funds the mission, teaches the framework, and builds trust through useful rights-cleared products.</x:v>
+      </x:c>
     </x:row>
     <x:row r="10">
       <x:c r="A10" s="50" t="str">
@@ -5337,6 +5395,12 @@
       <x:c r="F10" s="50" t="str">
         <x:v>Keep full PDF out of public GitHub; citation, quotation, image, trademark, accessibility, and distribution review.</x:v>
       </x:c>
+      <x:c r="G10" s="50" t="str">
+        <x:v>Sourced paper or brief, then paid talks, workshops, consulting, licensing, or a reader-facing book after review.</x:v>
+      </x:c>
+      <x:c r="H10" s="50" t="str">
+        <x:v>Portfolio support: preserves provenance, strengthens evidence, or supports delivery without overstating readiness.</x:v>
+      </x:c>
     </x:row>
     <x:row r="11">
       <x:c r="A11" s="50" t="str">
@@ -5357,6 +5421,12 @@
       <x:c r="F11" s="50" t="str">
         <x:v>Consolidate repeated drafts; ground claims in primary/scholarly sources; Black-studies, African-history, legal, and sensitivity review.</x:v>
       </x:c>
+      <x:c r="G11" s="50" t="str">
+        <x:v>Rights-cleared print, ebook, audiobook, music, or serialized edition after professional editing and launch preparation.</x:v>
+      </x:c>
+      <x:c r="H11" s="50" t="str">
+        <x:v>Portfolio support: preserves provenance, strengthens evidence, or supports delivery without overstating readiness.</x:v>
+      </x:c>
     </x:row>
     <x:row r="12">
       <x:c r="A12" s="50" t="str">
@@ -5377,6 +5447,12 @@
       <x:c r="F12" s="50" t="str">
         <x:v>Preserve unchanged; keep outside public GitHub and marketing; route only through authorized legal/agency channels.</x:v>
       </x:c>
+      <x:c r="G12" s="50" t="str">
+        <x:v>Package after audience, rights, evidence, safety, and delivery format are defined.</x:v>
+      </x:c>
+      <x:c r="H12" s="50" t="str">
+        <x:v>Portfolio support: preserves provenance, strengthens evidence, or supports delivery without overstating readiness.</x:v>
+      </x:c>
     </x:row>
     <x:row r="13">
       <x:c r="A13" s="50" t="str">
@@ -5397,6 +5473,12 @@
       <x:c r="F13" s="50" t="str">
         <x:v>Confirm contributions and metadata; create an accessible clean lead sheet; music-rights review before distribution.</x:v>
       </x:c>
+      <x:c r="G13" s="50" t="str">
+        <x:v>Rights-cleared print, ebook, audiobook, music, or serialized edition after professional editing and launch preparation.</x:v>
+      </x:c>
+      <x:c r="H13" s="50" t="str">
+        <x:v>Audience and revenue: funds the mission, teaches the framework, and builds trust through useful rights-cleared products.</x:v>
+      </x:c>
     </x:row>
     <x:row r="14">
       <x:c r="A14" s="50" t="str">
@@ -5417,6 +5499,12 @@
       <x:c r="F14" s="50" t="str">
         <x:v>Keep checksum/provenance; designate descriptive filename canonical; exclude from work/publication counts.</x:v>
       </x:c>
+      <x:c r="G14" s="50" t="str">
+        <x:v>Package after audience, rights, evidence, safety, and delivery format are defined.</x:v>
+      </x:c>
+      <x:c r="H14" s="50" t="str">
+        <x:v>Portfolio support: preserves provenance, strengthens evidence, or supports delivery without overstating readiness.</x:v>
+      </x:c>
     </x:row>
     <x:row r="15">
       <x:c r="A15" s="50" t="str">
@@ -5437,6 +5525,12 @@
       <x:c r="F15" s="50" t="str">
         <x:v>Preserve originals and chain of custody; do not rewrite evidence; share only with authorized recipients.</x:v>
       </x:c>
+      <x:c r="G15" s="50" t="str">
+        <x:v>Package after audience, rights, evidence, safety, and delivery format are defined.</x:v>
+      </x:c>
+      <x:c r="H15" s="50" t="str">
+        <x:v>Portfolio support: preserves provenance, strengthens evidence, or supports delivery without overstating readiness.</x:v>
+      </x:c>
     </x:row>
     <x:row r="16">
       <x:c r="A16" s="50" t="str">
@@ -5457,6 +5551,12 @@
       <x:c r="F16" s="50" t="str">
         <x:v>Complete structure and citations; define bounded tasks/failure metrics; public-safety, accessibility, cyber, privacy, labor, legal, and human-factors review.</x:v>
       </x:c>
+      <x:c r="G16" s="50" t="str">
+        <x:v>Sourced paper or brief, then paid talks, workshops, consulting, licensing, or a reader-facing book after review.</x:v>
+      </x:c>
+      <x:c r="H16" s="50" t="str">
+        <x:v>Portfolio support: preserves provenance, strengthens evidence, or supports delivery without overstating readiness.</x:v>
+      </x:c>
     </x:row>
     <x:row r="17">
       <x:c r="A17" s="50" t="str">
@@ -5477,6 +5577,12 @@
       <x:c r="F17" s="50" t="str">
         <x:v>Remove conversational scaffolding; verify citations; separate lived experience from general claims; Black-feminist/public-health review.</x:v>
       </x:c>
+      <x:c r="G17" s="50" t="str">
+        <x:v>Sourced paper or brief, then paid talks, workshops, consulting, licensing, or a reader-facing book after review.</x:v>
+      </x:c>
+      <x:c r="H17" s="50" t="str">
+        <x:v>Portfolio support: preserves provenance, strengthens evidence, or supports delivery without overstating readiness.</x:v>
+      </x:c>
     </x:row>
     <x:row r="18">
       <x:c r="A18" s="50" t="str">
@@ -5497,6 +5603,12 @@
       <x:c r="F18" s="50" t="str">
         <x:v>Separate memoir, satire, policy claims, and fiction; fact-check; edit for audience; legal and sensitivity review.</x:v>
       </x:c>
+      <x:c r="G18" s="50" t="str">
+        <x:v>Sourced paper or brief, then paid talks, workshops, consulting, licensing, or a reader-facing book after review.</x:v>
+      </x:c>
+      <x:c r="H18" s="50" t="str">
+        <x:v>Portfolio support: preserves provenance, strengthens evidence, or supports delivery without overstating readiness.</x:v>
+      </x:c>
     </x:row>
     <x:row r="19">
       <x:c r="A19" s="50" t="str">
@@ -5517,6 +5629,12 @@
       <x:c r="F19" s="50" t="str">
         <x:v>Check names/handles; research permits, insurance, food, welfare, zoonotic risk, accessibility, and venue rules; demand tests first.</x:v>
       </x:c>
+      <x:c r="G19" s="50" t="str">
+        <x:v>Package after audience, rights, evidence, safety, and delivery format are defined.</x:v>
+      </x:c>
+      <x:c r="H19" s="50" t="str">
+        <x:v>Portfolio support: preserves provenance, strengthens evidence, or supports delivery without overstating readiness.</x:v>
+      </x:c>
     </x:row>
     <x:row r="20">
       <x:c r="A20" s="50" t="str">
@@ -5537,6 +5655,12 @@
       <x:c r="F20" s="50" t="str">
         <x:v>Freeze unverified claims; prior-art/standards review; credentialed herpetology, veterinary, welfare, engineering, liability, and field-safety review.</x:v>
       </x:c>
+      <x:c r="G20" s="50" t="str">
+        <x:v>Prior art → requirements → simulation/bench proof → safety review → prototype → pilot → manufacturing → truthful launch.</x:v>
+      </x:c>
+      <x:c r="H20" s="50" t="str">
+        <x:v>Physical proof: turns claims into measured prototypes, independent review, production evidence, and useful products.</x:v>
+      </x:c>
     </x:row>
     <x:row r="21">
       <x:c r="A21" s="50" t="str">
@@ -5557,6 +5681,12 @@
       <x:c r="F21" s="50" t="str">
         <x:v>Jurisdictional feasibility: separation, permits, veterinary oversight, welfare, sanitation, zoonotic risk, insurance, accessibility, staffing, capital, and pilot alternatives.</x:v>
       </x:c>
+      <x:c r="G21" s="50" t="str">
+        <x:v>Private venture validation and partner outreach; sanitized prospectus only if useful.</x:v>
+      </x:c>
+      <x:c r="H21" s="50" t="str">
+        <x:v>Portfolio support: preserves provenance, strengthens evidence, or supports delivery without overstating readiness.</x:v>
+      </x:c>
     </x:row>
     <x:row r="22">
       <x:c r="A22" s="50" t="str">
@@ -5577,6 +5707,12 @@
       <x:c r="F22" s="50" t="str">
         <x:v>Combine base and supplement; verify DOI/doctrine citations; transformative-use, trademark, quotation, legal, and editorial review.</x:v>
       </x:c>
+      <x:c r="G22" s="50" t="str">
+        <x:v>Sourced paper or brief, then paid talks, workshops, consulting, licensing, or a reader-facing book after review.</x:v>
+      </x:c>
+      <x:c r="H22" s="50" t="str">
+        <x:v>Physical proof: turns claims into measured prototypes, independent review, production evidence, and useful products.</x:v>
+      </x:c>
     </x:row>
     <x:row r="23">
       <x:c r="A23" s="50" t="str">
@@ -5597,6 +5733,12 @@
       <x:c r="F23" s="50" t="str">
         <x:v>Japan visa/entity/licensing, food safety, alcohol rules if applicable, localization, demand, capital, unit economics, local legal/accounting review.</x:v>
       </x:c>
+      <x:c r="G23" s="50" t="str">
+        <x:v>Private venture validation and partner outreach; sanitized prospectus only if useful.</x:v>
+      </x:c>
+      <x:c r="H23" s="50" t="str">
+        <x:v>Portfolio support: preserves provenance, strengthens evidence, or supports delivery without overstating readiness.</x:v>
+      </x:c>
     </x:row>
     <x:row r="24">
       <x:c r="A24" s="50" t="str">
@@ -5617,6 +5759,12 @@
       <x:c r="F24" s="50" t="str">
         <x:v>Keep full manuscript private; audit canon, quotes, recipes, names, images, credits, trademarks, and commercial fan-work rights.</x:v>
       </x:c>
+      <x:c r="G24" s="50" t="str">
+        <x:v>Rights-cleared print, ebook, audiobook, music, or serialized edition after professional editing and launch preparation.</x:v>
+      </x:c>
+      <x:c r="H24" s="50" t="str">
+        <x:v>Audience and revenue: funds the mission, teaches the framework, and builds trust through useful rights-cleared products.</x:v>
+      </x:c>
     </x:row>
     <x:row r="25">
       <x:c r="A25" s="50" t="str">
@@ -5637,6 +5785,12 @@
       <x:c r="F25" s="50" t="str">
         <x:v>Exact dataset/license; preregistration; code/environment/checksums; negative controls; multiple-comparison/selection-bias tests; independent statistics/domain review.</x:v>
       </x:c>
+      <x:c r="G25" s="50" t="str">
+        <x:v>Sourced paper or brief, then paid talks, workshops, consulting, licensing, or a reader-facing book after review.</x:v>
+      </x:c>
+      <x:c r="H25" s="50" t="str">
+        <x:v>Portfolio support: preserves provenance, strengthens evidence, or supports delivery without overstating readiness.</x:v>
+      </x:c>
     </x:row>
     <x:row r="26">
       <x:c r="A26" s="50" t="str">
@@ -5657,6 +5811,12 @@
       <x:c r="F26" s="50" t="str">
         <x:v>Washington licensing, zoning, insurance, age controls, service duties, tasting rules, supplier economics, rent, turns, margin, capital, demand.</x:v>
       </x:c>
+      <x:c r="G26" s="50" t="str">
+        <x:v>Private venture validation and partner outreach; sanitized prospectus only if useful.</x:v>
+      </x:c>
+      <x:c r="H26" s="50" t="str">
+        <x:v>Portfolio support: preserves provenance, strengthens evidence, or supports delivery without overstating readiness.</x:v>
+      </x:c>
     </x:row>
     <x:row r="27">
       <x:c r="A27" s="50" t="str">
@@ -5677,6 +5837,12 @@
       <x:c r="F27" s="50" t="str">
         <x:v>Record URL/capture date; current official version and qualified immigration advice; quote narrowly with attribution; do not upload full copy.</x:v>
       </x:c>
+      <x:c r="G27" s="50" t="str">
+        <x:v>Archive or protected source only; no direct sale.</x:v>
+      </x:c>
+      <x:c r="H27" s="50" t="str">
+        <x:v>Physical proof: turns claims into measured prototypes, independent review, production evidence, and useful products.</x:v>
+      </x:c>
     </x:row>
     <x:row r="28">
       <x:c r="A28" s="50" t="str">
@@ -5697,6 +5863,12 @@
       <x:c r="F28" s="50" t="str">
         <x:v>Separate original commentary from third-party setting/marks; rights/editorial review; develop rights-cleared original-city version.</x:v>
       </x:c>
+      <x:c r="G28" s="50" t="str">
+        <x:v>Rights-cleared print, ebook, audiobook, music, or serialized edition after professional editing and launch preparation.</x:v>
+      </x:c>
+      <x:c r="H28" s="50" t="str">
+        <x:v>Accountability practice: converts system failures into auditable methods, training, paid services, and institutional repair tools.</x:v>
+      </x:c>
     </x:row>
     <x:row r="29">
       <x:c r="A29" s="50" t="str">
@@ -5717,6 +5889,12 @@
       <x:c r="F29" s="50" t="str">
         <x:v>Protect health/legal/housing details; do not publish raw dialogue; verify claims; legal/medical support as appropriate; separate anonymized essay after review.</x:v>
       </x:c>
+      <x:c r="G29" s="50" t="str">
+        <x:v>Sourced paper or brief, then paid talks, workshops, consulting, licensing, or a reader-facing book after review.</x:v>
+      </x:c>
+      <x:c r="H29" s="50" t="str">
+        <x:v>Portfolio support: preserves provenance, strengthens evidence, or supports delivery without overstating readiness.</x:v>
+      </x:c>
     </x:row>
     <x:row r="30">
       <x:c r="A30" s="50" t="str">
@@ -5737,6 +5915,12 @@
       <x:c r="F30" s="50" t="str">
         <x:v>Verify citations/quotes; refine terminology; historians of religion, Indigenous history, colonial studies, and sensitivity review.</x:v>
       </x:c>
+      <x:c r="G30" s="50" t="str">
+        <x:v>Sourced paper or brief, then paid talks, workshops, consulting, licensing, or a reader-facing book after review.</x:v>
+      </x:c>
+      <x:c r="H30" s="50" t="str">
+        <x:v>Portfolio support: preserves provenance, strengthens evidence, or supports delivery without overstating readiness.</x:v>
+      </x:c>
     </x:row>
     <x:row r="31">
       <x:c r="A31" s="50" t="str">
@@ -5757,6 +5941,12 @@
       <x:c r="F31" s="50" t="str">
         <x:v>Merge/cross-reference as supplement; verify DOI live; preserve lineage; avoid double-counting.</x:v>
       </x:c>
+      <x:c r="G31" s="50" t="str">
+        <x:v>Package after audience, rights, evidence, safety, and delivery format are defined.</x:v>
+      </x:c>
+      <x:c r="H31" s="50" t="str">
+        <x:v>Portfolio support: preserves provenance, strengthens evidence, or supports delivery without overstating readiness.</x:v>
+      </x:c>
     </x:row>
     <x:row r="32">
       <x:c r="A32" s="50" t="str">
@@ -5777,6 +5967,12 @@
       <x:c r="F32" s="50" t="str">
         <x:v>Bound assertions; cited readings; learner safeguards; accessibility; rubrics; legal/trauma-aware review; supervised pilot.</x:v>
       </x:c>
+      <x:c r="G32" s="50" t="str">
+        <x:v>Rights-cleared workbook, facilitator kit, cohort course, institutional license, or consulting package after review and pilot evidence.</x:v>
+      </x:c>
+      <x:c r="H32" s="50" t="str">
+        <x:v>Portfolio support: preserves provenance, strengthens evidence, or supports delivery without overstating readiness.</x:v>
+      </x:c>
     </x:row>
     <x:row r="33">
       <x:c r="A33" s="50" t="str">
@@ -5797,6 +5993,12 @@
       <x:c r="F33" s="50" t="str">
         <x:v>Bound categorical claims; add emergency/legal/disability/referral guidance; test with tenants, caseworkers, and legal reviewers.</x:v>
       </x:c>
+      <x:c r="G33" s="50" t="str">
+        <x:v>Rights-cleared workbook, facilitator kit, cohort course, institutional license, or consulting package after review and pilot evidence.</x:v>
+      </x:c>
+      <x:c r="H33" s="50" t="str">
+        <x:v>Audience and revenue: funds the mission, teaches the framework, and builds trust through useful rights-cleared products.</x:v>
+      </x:c>
     </x:row>
     <x:row r="34">
       <x:c r="A34" s="50" t="str">
@@ -5817,6 +6019,12 @@
       <x:c r="F34" s="50" t="str">
         <x:v>Validate model; add context, exceptions, legal-record duties, escalation routes, and warnings against withholding material facts.</x:v>
       </x:c>
+      <x:c r="G34" s="50" t="str">
+        <x:v>Rights-cleared workbook, facilitator kit, cohort course, institutional license, or consulting package after review and pilot evidence.</x:v>
+      </x:c>
+      <x:c r="H34" s="50" t="str">
+        <x:v>Portfolio support: preserves provenance, strengthens evidence, or supports delivery without overstating readiness.</x:v>
+      </x:c>
     </x:row>
     <x:row r="35">
       <x:c r="A35" s="50" t="str">
@@ -5837,6 +6045,12 @@
       <x:c r="F35" s="50" t="str">
         <x:v>Canonicalize; merge guide/map appendices; source claims; jurisdiction/crisis disclaimers; accessibility/legal/usability review.</x:v>
       </x:c>
+      <x:c r="G35" s="50" t="str">
+        <x:v>Rights-cleared workbook, facilitator kit, cohort course, institutional license, or consulting package after review and pilot evidence.</x:v>
+      </x:c>
+      <x:c r="H35" s="50" t="str">
+        <x:v>Audience and revenue: funds the mission, teaches the framework, and builds trust through useful rights-cleared products.</x:v>
+      </x:c>
     </x:row>
     <x:row r="36">
       <x:c r="A36" s="50" t="str">
@@ -5857,6 +6071,12 @@
       <x:c r="F36" s="50" t="str">
         <x:v>Select canonical version; preserve lineage; verify citations/case claims; distinguish hypotheses; independent systems/legal/public-administration review.</x:v>
       </x:c>
+      <x:c r="G36" s="50" t="str">
+        <x:v>Sourced paper or brief, then paid talks, workshops, consulting, licensing, or a reader-facing book after review.</x:v>
+      </x:c>
+      <x:c r="H36" s="50" t="str">
+        <x:v>Portfolio support: preserves provenance, strengthens evidence, or supports delivery without overstating readiness.</x:v>
+      </x:c>
     </x:row>
     <x:row r="37">
       <x:c r="A37" s="50" t="str">
@@ -5877,6 +6097,12 @@
       <x:c r="F37" s="50" t="str">
         <x:v>Diff against canonical; protect personal case appendix; retain unique theory with provenance; no raw identifying facts.</x:v>
       </x:c>
+      <x:c r="G37" s="50" t="str">
+        <x:v>Package after audience, rights, evidence, safety, and delivery format are defined.</x:v>
+      </x:c>
+      <x:c r="H37" s="50" t="str">
+        <x:v>Portfolio support: preserves provenance, strengthens evidence, or supports delivery without overstating readiness.</x:v>
+      </x:c>
     </x:row>
     <x:row r="38">
       <x:c r="A38" s="50" t="str">
@@ -5897,6 +6123,12 @@
       <x:c r="F38" s="50" t="str">
         <x:v>Split general paper from personal/legal evidence; audit citations/claims; ethics, legal, critical-race, and public-administration review.</x:v>
       </x:c>
+      <x:c r="G38" s="50" t="str">
+        <x:v>Sourced paper or brief, then paid talks, workshops, consulting, licensing, or a reader-facing book after review.</x:v>
+      </x:c>
+      <x:c r="H38" s="50" t="str">
+        <x:v>Portfolio support: preserves provenance, strengthens evidence, or supports delivery without overstating readiness.</x:v>
+      </x:c>
     </x:row>
     <x:row r="39">
       <x:c r="A39" s="50" t="str">
@@ -5917,6 +6149,12 @@
       <x:c r="F39" s="50" t="str">
         <x:v>Do not count; retain checksum only if provenance matters, otherwise archive outside active portfolio.</x:v>
       </x:c>
+      <x:c r="G39" s="50" t="str">
+        <x:v>Archive or protected source only; no direct sale.</x:v>
+      </x:c>
+      <x:c r="H39" s="50" t="str">
+        <x:v>Portfolio support: preserves provenance, strengthens evidence, or supports delivery without overstating readiness.</x:v>
+      </x:c>
     </x:row>
     <x:row r="40">
       <x:c r="A40" s="50" t="str">
@@ -5937,6 +6175,12 @@
       <x:c r="F40" s="50" t="str">
         <x:v>Map canonical filenames, versions, evidence levels, public/private status, citations, dependencies, and missing artifacts; sanitize case details.</x:v>
       </x:c>
+      <x:c r="G40" s="50" t="str">
+        <x:v>Package after audience, rights, evidence, safety, and delivery format are defined.</x:v>
+      </x:c>
+      <x:c r="H40" s="50" t="str">
+        <x:v>Physical proof: turns claims into measured prototypes, independent review, production evidence, and useful products.</x:v>
+      </x:c>
     </x:row>
     <x:row r="41">
       <x:c r="A41" s="50" t="str">
@@ -5957,6 +6201,12 @@
       <x:c r="F41" s="50" t="str">
         <x:v>Bound and source claims; separate metaphor/evidence/lived experience/manifesto; multidisciplinary scholarly, sensitivity, and editorial review.</x:v>
       </x:c>
+      <x:c r="G41" s="50" t="str">
+        <x:v>Rights-cleared print, ebook, audiobook, music, or serialized edition after professional editing and launch preparation.</x:v>
+      </x:c>
+      <x:c r="H41" s="50" t="str">
+        <x:v>Public framework: builds the case for durable guardrails, shared reality, institutional memory, and stable self-governance.</x:v>
+      </x:c>
     </x:row>
     <x:row r="42">
       <x:c r="A42" s="50" t="str">
@@ -5977,6 +6227,12 @@
       <x:c r="F42" s="50" t="str">
         <x:v>Diff versions; designate canonical; source ledger; remove duplication/conversational residue; multidisciplinary review/edit.</x:v>
       </x:c>
+      <x:c r="G42" s="50" t="str">
+        <x:v>Rights-cleared print, ebook, audiobook, music, or serialized edition after professional editing and launch preparation.</x:v>
+      </x:c>
+      <x:c r="H42" s="50" t="str">
+        <x:v>Public framework: builds the case for durable guardrails, shared reality, institutional memory, and stable self-governance.</x:v>
+      </x:c>
     </x:row>
     <x:row r="43">
       <x:c r="A43" s="50" t="str">
@@ -5997,6 +6253,12 @@
       <x:c r="F43" s="50" t="str">
         <x:v>Keep evidence private; counsel verifies privilege/accuracy/retaliation/public-record risk; formal de-identification; methods/housing-law/ethics review.</x:v>
       </x:c>
+      <x:c r="G43" s="50" t="str">
+        <x:v>Sourced paper or brief, then paid talks, workshops, consulting, licensing, or a reader-facing book after review.</x:v>
+      </x:c>
+      <x:c r="H43" s="50" t="str">
+        <x:v>Accountability practice: converts system failures into auditable methods, training, paid services, and institutional repair tools.</x:v>
+      </x:c>
     </x:row>
     <x:row r="44">
       <x:c r="A44" s="50" t="str">
@@ -6017,6 +6279,12 @@
       <x:c r="F44" s="50" t="str">
         <x:v>Verify regulations/data/citations; calibrate design claims; separate general theory from case inference; multidisciplinary review.</x:v>
       </x:c>
+      <x:c r="G44" s="50" t="str">
+        <x:v>Sourced paper or brief, then paid talks, workshops, consulting, licensing, or a reader-facing book after review.</x:v>
+      </x:c>
+      <x:c r="H44" s="50" t="str">
+        <x:v>Physical proof: turns claims into measured prototypes, independent review, production evidence, and useful products.</x:v>
+      </x:c>
     </x:row>
     <x:row r="45">
       <x:c r="A45" s="50" t="str">
@@ -6037,6 +6305,12 @@
       <x:c r="F45" s="50" t="str">
         <x:v>Operationalize scope; source claims; distinguish design/incentive/outcome; add counterexamples/falsification; systems/economics/history/policy review.</x:v>
       </x:c>
+      <x:c r="G45" s="50" t="str">
+        <x:v>Sourced paper or brief, then paid talks, workshops, consulting, licensing, or a reader-facing book after review.</x:v>
+      </x:c>
+      <x:c r="H45" s="50" t="str">
+        <x:v>Public framework: builds the case for durable guardrails, shared reality, institutional memory, and stable self-governance.</x:v>
+      </x:c>
     </x:row>
     <x:row r="46">
       <x:c r="A46" s="50" t="str">
@@ -6057,6 +6331,12 @@
       <x:c r="F46" s="50" t="str">
         <x:v>Preserve correspondence; verify quotes/chronology; counsel review names/allegations; anonymize theory; no identifying evidence publication.</x:v>
       </x:c>
+      <x:c r="G46" s="50" t="str">
+        <x:v>Sourced paper or brief, then paid talks, workshops, consulting, licensing, or a reader-facing book after review.</x:v>
+      </x:c>
+      <x:c r="H46" s="50" t="str">
+        <x:v>Accountability practice: converts system failures into auditable methods, training, paid services, and institutional repair tools.</x:v>
+      </x:c>
     </x:row>
     <x:row r="47">
       <x:c r="A47" s="50" t="str">
@@ -6077,6 +6357,12 @@
       <x:c r="F47" s="50" t="str">
         <x:v>Validate mechanism or label conceptual; citations, counter-hypotheses, limitations; ethics/critical-race/AI/access/legal review.</x:v>
       </x:c>
+      <x:c r="G47" s="50" t="str">
+        <x:v>Sourced paper or brief, then paid talks, workshops, consulting, licensing, or a reader-facing book after review.</x:v>
+      </x:c>
+      <x:c r="H47" s="50" t="str">
+        <x:v>Physical proof: turns claims into measured prototypes, independent review, production evidence, and useful products.</x:v>
+      </x:c>
     </x:row>
     <x:row r="48">
       <x:c r="A48" s="50" t="str">
@@ -6097,6 +6383,12 @@
       <x:c r="F48" s="50" t="str">
         <x:v>Choose genre; source claims; add limitations; legal, historical, critical-race, and editorial review.</x:v>
       </x:c>
+      <x:c r="G48" s="50" t="str">
+        <x:v>Sourced paper or brief, then paid talks, workshops, consulting, licensing, or a reader-facing book after review.</x:v>
+      </x:c>
+      <x:c r="H48" s="50" t="str">
+        <x:v>Portfolio support: preserves provenance, strengthens evidence, or supports delivery without overstating readiness.</x:v>
+      </x:c>
     </x:row>
     <x:row r="49">
       <x:c r="A49" s="50" t="str">
@@ -6117,6 +6409,12 @@
       <x:c r="F49" s="50" t="str">
         <x:v>Canonicalize; remove private ending; verify medical/mortality claims; no individual diagnosis; epidemiology/housing-health/clinical/legal/ethics review.</x:v>
       </x:c>
+      <x:c r="G49" s="50" t="str">
+        <x:v>Sourced paper or brief, then paid talks, workshops, consulting, licensing, or a reader-facing book after review.</x:v>
+      </x:c>
+      <x:c r="H49" s="50" t="str">
+        <x:v>Accountability practice: converts system failures into auditable methods, training, paid services, and institutional repair tools.</x:v>
+      </x:c>
     </x:row>
     <x:row r="50">
       <x:c r="A50" s="50" t="str">
@@ -6137,6 +6435,12 @@
       <x:c r="F50" s="50" t="str">
         <x:v>Retain checksum/provenance; consolidate under canonical title; exclude from counts.</x:v>
       </x:c>
+      <x:c r="G50" s="50" t="str">
+        <x:v>Package after audience, rights, evidence, safety, and delivery format are defined.</x:v>
+      </x:c>
+      <x:c r="H50" s="50" t="str">
+        <x:v>Accountability practice: converts system failures into auditable methods, training, paid services, and institutional repair tools.</x:v>
+      </x:c>
     </x:row>
     <x:row r="51">
       <x:c r="A51" s="50" t="str">
@@ -6157,6 +6461,12 @@
       <x:c r="F51" s="50" t="str">
         <x:v>Verify mechanisms against agreements/ledgers/rules/law/accounting; separate case from prevalence; counsel/accountant/methods/tenant review.</x:v>
       </x:c>
+      <x:c r="G51" s="50" t="str">
+        <x:v>Sourced paper or brief, then paid talks, workshops, consulting, licensing, or a reader-facing book after review.</x:v>
+      </x:c>
+      <x:c r="H51" s="50" t="str">
+        <x:v>Accountability practice: converts system failures into auditable methods, training, paid services, and institutional repair tools.</x:v>
+      </x:c>
     </x:row>
     <x:row r="52">
       <x:c r="A52" s="50" t="str">
@@ -6177,6 +6487,12 @@
       <x:c r="F52" s="50" t="str">
         <x:v>Keep identifying evidence private; preserve originals; housing counsel/accounting review; separately de-identified teaching edition only with consent and ethics review.</x:v>
       </x:c>
+      <x:c r="G52" s="50" t="str">
+        <x:v>Rights-cleared workbook, facilitator kit, cohort course, institutional license, or consulting package after review and pilot evidence.</x:v>
+      </x:c>
+      <x:c r="H52" s="50" t="str">
+        <x:v>Accountability practice: converts system failures into auditable methods, training, paid services, and institutional repair tools.</x:v>
+      </x:c>
     </x:row>
     <x:row r="53">
       <x:c r="A53" s="50" t="str">
@@ -6197,6 +6513,12 @@
       <x:c r="F53" s="50" t="str">
         <x:v>Never place on public GitHub; preserve chain of custody/hash; restrict access; counsel controls disclosure, redaction, and derivative use.</x:v>
       </x:c>
+      <x:c r="G53" s="50" t="str">
+        <x:v>Archive or protected source only; no direct sale.</x:v>
+      </x:c>
+      <x:c r="H53" s="50" t="str">
+        <x:v>Accountability practice: converts system failures into auditable methods, training, paid services, and institutional repair tools.</x:v>
+      </x:c>
     </x:row>
     <x:row r="54">
       <x:c r="A54" s="50" t="str">
@@ -6217,6 +6539,12 @@
       <x:c r="F54" s="50" t="str">
         <x:v>Do not count; retain checksum only if provenance matters, otherwise archive outside active portfolio.</x:v>
       </x:c>
+      <x:c r="G54" s="50" t="str">
+        <x:v>Archive or protected source only; no direct sale.</x:v>
+      </x:c>
+      <x:c r="H54" s="50" t="str">
+        <x:v>Portfolio support: preserves provenance, strengthens evidence, or supports delivery without overstating readiness.</x:v>
+      </x:c>
     </x:row>
     <x:row r="55">
       <x:c r="A55" s="50" t="str">
@@ -6237,6 +6565,12 @@
       <x:c r="F55" s="50" t="str">
         <x:v>Define metaphor/scope; verify every table/statistic with primary sources; remove residue; Black feminist/public-health/legal/statistical/community review.</x:v>
       </x:c>
+      <x:c r="G55" s="50" t="str">
+        <x:v>Sourced paper or brief, then paid talks, workshops, consulting, licensing, or a reader-facing book after review.</x:v>
+      </x:c>
+      <x:c r="H55" s="50" t="str">
+        <x:v>Portfolio support: preserves provenance, strengthens evidence, or supports delivery without overstating readiness.</x:v>
+      </x:c>
     </x:row>
     <x:row r="56">
       <x:c r="A56" s="50" t="str">
@@ -6257,6 +6591,12 @@
       <x:c r="F56" s="50" t="str">
         <x:v>Remove chat residue; specify governance, consent, minimization, correction, access, retention, de-identification, and community oversight; privacy-safe pilot.</x:v>
       </x:c>
+      <x:c r="G56" s="50" t="str">
+        <x:v>Package after audience, rights, evidence, safety, and delivery format are defined.</x:v>
+      </x:c>
+      <x:c r="H56" s="50" t="str">
+        <x:v>Accountability practice: converts system failures into auditable methods, training, paid services, and institutional repair tools.</x:v>
+      </x:c>
     </x:row>
     <x:row r="57">
       <x:c r="A57" s="50" t="str">
@@ -6277,6 +6617,12 @@
       <x:c r="F57" s="50" t="str">
         <x:v>Use as appendix; remove personal dialogue and unsupported assertions; publish only rights-cleared, sourced analysis.</x:v>
       </x:c>
+      <x:c r="G57" s="50" t="str">
+        <x:v>Package after audience, rights, evidence, safety, and delivery format are defined.</x:v>
+      </x:c>
+      <x:c r="H57" s="50" t="str">
+        <x:v>Portfolio support: preserves provenance, strengthens evidence, or supports delivery without overstating readiness.</x:v>
+      </x:c>
     </x:row>
     <x:row r="58">
       <x:c r="A58" s="50" t="str">
@@ -6297,6 +6643,12 @@
       <x:c r="F58" s="50" t="str">
         <x:v>Verify examples; define mechanisms/falsification; separate analogy from evidence; rights review fictional references; history/governance/editorial review.</x:v>
       </x:c>
+      <x:c r="G58" s="50" t="str">
+        <x:v>Package after audience, rights, evidence, safety, and delivery format are defined.</x:v>
+      </x:c>
+      <x:c r="H58" s="50" t="str">
+        <x:v>Public framework: builds the case for durable guardrails, shared reality, institutional memory, and stable self-governance.</x:v>
+      </x:c>
     </x:row>
     <x:row r="59">
       <x:c r="A59" s="50" t="str">
@@ -6317,31 +6669,303 @@
       <x:c r="F59" s="50" t="str">
         <x:v>Keep planning private; verify role/credential claims; create separate sanitized resume, portfolio summary, and role-target matrix.</x:v>
       </x:c>
+      <x:c r="G59" s="50" t="str">
+        <x:v>Package after audience, rights, evidence, safety, and delivery format are defined.</x:v>
+      </x:c>
+      <x:c r="H59" s="50" t="str">
+        <x:v>Portfolio support: preserves provenance, strengthens evidence, or supports delivery without overstating readiness.</x:v>
+      </x:c>
     </x:row>
     <x:row r="60">
-      <x:c r="A60" s="51" t="str">
+      <x:c r="A60" s="50" t="str">
         <x:v>A Longitudinal Analysis of Human Reform, Regression, and Relapse</x:v>
       </x:c>
-      <x:c r="B60" s="51" t="str">
+      <x:c r="B60" s="50" t="str">
         <x:v>Historical systems-analysis addendum</x:v>
       </x:c>
-      <x:c r="C60" s="51" t="str">
+      <x:c r="C60" s="50" t="str">
         <x:v>Public candidate after rigorous historical review</x:v>
       </x:c>
-      <x:c r="D60" s="51" t="str">
+      <x:c r="D60" s="50" t="str">
         <x:v>Addendum D</x:v>
       </x:c>
-      <x:c r="E60" s="51" t="str">
+      <x:c r="E60" s="50" t="str">
         <x:v>Historical cycle and learning-retention scale for reform, regression, relapse, and institutional memory.</x:v>
       </x:c>
-      <x:c r="F60" s="51" t="str">
+      <x:c r="F60" s="50" t="str">
         <x:v>Operationalize scale; predefine cases/coding; test counterexamples; calibrate claims; sources and history/comparative-politics/methods review.</x:v>
+      </x:c>
+      <x:c r="G60" s="50" t="str">
+        <x:v>Package after audience, rights, evidence, safety, and delivery format are defined.</x:v>
+      </x:c>
+      <x:c r="H60" s="50" t="str">
+        <x:v>Public framework: builds the case for durable guardrails, shared reality, institutional memory, and stable self-governance.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="61">
+      <x:c r="A61" s="50" t="str">
+        <x:v>How to Fix Us — A Systems-Level Treatment Framework for Stable Self-Governance</x:v>
+      </x:c>
+      <x:c r="B61" s="50" t="str">
+        <x:v>Civilizational systems book and policy framework</x:v>
+      </x:c>
+      <x:c r="C61" s="50" t="str">
+        <x:v>Public book/policy-brief candidate after source/governance review</x:v>
+      </x:c>
+      <x:c r="D61" s="50" t="str">
+        <x:v>Paired treatment volume in human-sanity family</x:v>
+      </x:c>
+      <x:c r="E61" s="50" t="str">
+        <x:v>Five-shift treatment framework on guardrails, power constraints, structural memory, human-flaw design, and rejection of savior narratives.</x:v>
+      </x:c>
+      <x:c r="F61" s="50" t="str">
+        <x:v>Merge duplicate Part II; verify sources/policy examples; separate proposals from tested interventions; add tradeoffs/limits; multidisciplinary review.</x:v>
+      </x:c>
+      <x:c r="G61" s="50" t="str">
+        <x:v>Rights-cleared print, ebook, audiobook, music, or serialized edition after professional editing and launch preparation.</x:v>
+      </x:c>
+      <x:c r="H61" s="50" t="str">
+        <x:v>Public framework: builds the case for durable guardrails, shared reality, institutional memory, and stable self-governance.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="62">
+      <x:c r="A62" s="50" t="str">
+        <x:v>WTF Is Wrong With Us — A Systems-Level Analysis of Human Sanity, Risk, and Self-Regulation</x:v>
+      </x:c>
+      <x:c r="B62" s="50" t="str">
+        <x:v>Civilizational systems book and research essay</x:v>
+      </x:c>
+      <x:c r="C62" s="50" t="str">
+        <x:v>Public book candidate after evidence/tone/sensitivity review</x:v>
+      </x:c>
+      <x:c r="D62" s="50" t="str">
+        <x:v>Diagnosis volume paired with How to Fix Us</x:v>
+      </x:c>
+      <x:c r="E62" s="50" t="str">
+        <x:v>Diagnosis of collective self-harm, institutional abstraction, risk amplification, reform relapse, and the gap between technical power and ethical constraint.</x:v>
+      </x:c>
+      <x:c r="F62" s="50" t="str">
+        <x:v>Remove dialogue scaffolding; keep species diagnosis metaphorical; verify citations; define sanity index as illustrative; add counterevidence/limits; expert review.</x:v>
+      </x:c>
+      <x:c r="G62" s="50" t="str">
+        <x:v>Rights-cleared print, ebook, audiobook, music, or serialized edition after professional editing and launch preparation.</x:v>
+      </x:c>
+      <x:c r="H62" s="50" t="str">
+        <x:v>Public framework: builds the case for durable guardrails, shared reality, institutional memory, and stable self-governance.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="63">
+      <x:c r="A63" s="50" t="str">
+        <x:v>Aliens^.^.docx</x:v>
+      </x:c>
+      <x:c r="B63" s="50" t="str">
+        <x:v>Raw developmental conversation and source notebook</x:v>
+      </x:c>
+      <x:c r="C63" s="50" t="str">
+        <x:v>Private source; not market-ready</x:v>
+      </x:c>
+      <x:c r="D63" s="50" t="str">
+        <x:v>Support source — not separate work</x:v>
+      </x:c>
+      <x:c r="E63" s="50" t="str">
+        <x:v>Exploratory dialogue on alien metaphors, inhuman systems, civilizational risk, grounded reality testing, grief, accountability, and treatment frameworks.</x:v>
+      </x:c>
+      <x:c r="F63" s="50" t="str">
+        <x:v>Do not publish raw; extract original arguments with provenance; remove repetition/private material; use only as controlled source notebook.</x:v>
+      </x:c>
+      <x:c r="G63" s="50" t="str">
+        <x:v>Archive or protected source only; no direct sale.</x:v>
+      </x:c>
+      <x:c r="H63" s="50" t="str">
+        <x:v>Audience and revenue: funds the mission, teaches the framework, and builds trust through useful rights-cleared products.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="64">
+      <x:c r="A64" s="50" t="str">
+        <x:v>Starfleet Academy — Division of Governance, Systems Integrity and Accountability</x:v>
+      </x:c>
+      <x:c r="B64" s="50" t="str">
+        <x:v>Expanded fiction-framed curriculum/workbook/capstone system</x:v>
+      </x:c>
+      <x:c r="C64" s="50" t="str">
+        <x:v>Rights-restricted product; rights-cleared original edition recommended</x:v>
+      </x:c>
+      <x:c r="D64" s="50" t="str">
+        <x:v>Existing Starfleet Academy lineage — not separate work</x:v>
+      </x:c>
+      <x:c r="E64" s="50" t="str">
+        <x:v>Multi-volume governance/accountability program with syllabi, labs, simulations, workbooks, worksheets, capstone defense, binder, and low-energy tools.</x:v>
+      </x:c>
+      <x:c r="F64" s="50" t="str">
+        <x:v>Separate original pedagogy from third-party IP; remove fictional accreditation claims; verify readings; curriculum/accessibility/legal/rights/assessment review; rename.</x:v>
+      </x:c>
+      <x:c r="G64" s="50" t="str">
+        <x:v>Rights-cleared workbook, facilitator kit, cohort course, institutional license, or consulting package after review and pilot evidence.</x:v>
+      </x:c>
+      <x:c r="H64" s="50" t="str">
+        <x:v>Audience and revenue: funds the mission, teaches the framework, and builds trust through useful rights-cleared products.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="65">
+      <x:c r="A65" s="50" t="str">
+        <x:v>Accounting Curriculum Lab 3 — Clean Ledger Skeleton</x:v>
+      </x:c>
+      <x:c r="B65" s="50" t="str">
+        <x:v>Workbook lab and accounting-control template</x:v>
+      </x:c>
+      <x:c r="C65" s="50" t="str">
+        <x:v>Private training component; sanitized template sellable</x:v>
+      </x:c>
+      <x:c r="D65" s="50" t="str">
+        <x:v>Harm Without Awareness component — not separate work</x:v>
+      </x:c>
+      <x:c r="E65" s="50" t="str">
+        <x:v>Zero-entry monthly ledger, artifact index, permission rules, balance formula, and freeze logic for unresolved discrepancies.</x:v>
+      </x:c>
+      <x:c r="F65" s="50" t="str">
+        <x:v>Correct residue; validate accounting treatment; clearly fictional examples; accountant, housing-law, and curriculum usability review.</x:v>
+      </x:c>
+      <x:c r="G65" s="50" t="str">
+        <x:v>Rights-cleared workbook, facilitator kit, cohort course, institutional license, or consulting package after review and pilot evidence.</x:v>
+      </x:c>
+      <x:c r="H65" s="50" t="str">
+        <x:v>Accountability practice: converts system failures into auditable methods, training, paid services, and institutional repair tools.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="66">
+      <x:c r="A66" s="50" t="str">
+        <x:v>Harm Without Awareness — Training Modules for Others</x:v>
+      </x:c>
+      <x:c r="B66" s="50" t="str">
+        <x:v>Professional training-track architecture</x:v>
+      </x:c>
+      <x:c r="C66" s="50" t="str">
+        <x:v>Commercial curriculum component after review</x:v>
+      </x:c>
+      <x:c r="D66" s="50" t="str">
+        <x:v>STSAE curriculum component — not separate work</x:v>
+      </x:c>
+      <x:c r="E66" s="50" t="str">
+        <x:v>Three tiered tracks for tenants/advocates, investigators/compliance staff, and policy/audit leadership with applied capstones.</x:v>
+      </x:c>
+      <x:c r="F66" s="50" t="str">
+        <x:v>Expand lesson plans, facilitator notes, timing, assessment, accessibility, trauma safeguards, disclaimers, metrics; compensated community pilot.</x:v>
+      </x:c>
+      <x:c r="G66" s="50" t="str">
+        <x:v>Rights-cleared workbook, facilitator kit, cohort course, institutional license, or consulting package after review and pilot evidence.</x:v>
+      </x:c>
+      <x:c r="H66" s="50" t="str">
+        <x:v>Accountability practice: converts system failures into auditable methods, training, paid services, and institutional repair tools.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="67">
+      <x:c r="A67" s="50" t="str">
+        <x:v>When Enforcement Outruns Accounting</x:v>
+      </x:c>
+      <x:c r="B67" s="50" t="str">
+        <x:v>Housing accountability case study and training anchor</x:v>
+      </x:c>
+      <x:c r="C67" s="50" t="str">
+        <x:v>Strictly private case; de-identified publication candidate</x:v>
+      </x:c>
+      <x:c r="D67" s="50" t="str">
+        <x:v>Existing ledger-accountability family — not separate work</x:v>
+      </x:c>
+      <x:c r="E67" s="50" t="str">
+        <x:v>Case analysis of enforcement amid disputed accounting, rent-calculation error, repayment questions, and third-party funding requirements.</x:v>
+      </x:c>
+      <x:c r="F67" s="50" t="str">
+        <x:v>Preserve evidence; counsel verifies facts/quotes; separate allegation/admission/inference/recommendation; rigorously de-identified teaching case.</x:v>
+      </x:c>
+      <x:c r="G67" s="50" t="str">
+        <x:v>Rights-cleared workbook, facilitator kit, cohort course, institutional license, or consulting package after review and pilot evidence.</x:v>
+      </x:c>
+      <x:c r="H67" s="50" t="str">
+        <x:v>Accountability practice: converts system failures into auditable methods, training, paid services, and institutional repair tools.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="68">
+      <x:c r="A68" s="50" t="str">
+        <x:v>Human Dignity Is the Byproduct</x:v>
+      </x:c>
+      <x:c r="B68" s="50" t="str">
+        <x:v>Housing operations and incentive-design policy paper</x:v>
+      </x:c>
+      <x:c r="C68" s="50" t="str">
+        <x:v>Public brief/consulting candidate after evidence review</x:v>
+      </x:c>
+      <x:c r="D68" s="50" t="str">
+        <x:v>No match in recovered 60</x:v>
+      </x:c>
+      <x:c r="E68" s="50" t="str">
+        <x:v>Incentive-design argument that ledger clarity, early resolution, verified accounting, and outcome metrics can improve institutional results and resident dignity.</x:v>
+      </x:c>
+      <x:c r="F68" s="50" t="str">
+        <x:v>Test financial/behavioral claims; measurable hypotheses; cost model, metrics, failure cases, labor effects, implementation; multidisciplinary review.</x:v>
+      </x:c>
+      <x:c r="G68" s="50" t="str">
+        <x:v>Sourced paper or brief, then paid talks, workshops, consulting, licensing, or a reader-facing book after review.</x:v>
+      </x:c>
+      <x:c r="H68" s="50" t="str">
+        <x:v>Accountability practice: converts system failures into auditable methods, training, paid services, and institutional repair tools.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="69">
+      <x:c r="A69" s="50" t="str">
+        <x:v>Socio-Technical Systems Accountability Engineer — Harm Without Awareness</x:v>
+      </x:c>
+      <x:c r="B69" s="50" t="str">
+        <x:v>Professional field manual, curriculum, and service methodology</x:v>
+      </x:c>
+      <x:c r="C69" s="50" t="str">
+        <x:v>Flagship training/consulting candidate after completion/review</x:v>
+      </x:c>
+      <x:c r="D69" s="50" t="str">
+        <x:v>Canonical STSAE/Harm Without Awareness candidate</x:v>
+      </x:c>
+      <x:c r="E69" s="50" t="str">
+        <x:v>Manual defining the accountability-engineer role, artifact analysis, mechanism/effect statements, maps, counter-documentation, counter-design, and curriculum.</x:v>
+      </x:c>
+      <x:c r="F69" s="50" t="str">
+        <x:v>Replace placeholders; remove residue/absolutes; verify scholarship; examples, rubrics, ethics, scope, accessibility/legal boundaries; pilot and document outcomes.</x:v>
+      </x:c>
+      <x:c r="G69" s="50" t="str">
+        <x:v>Rights-cleared workbook, facilitator kit, cohort course, institutional license, or consulting package after review and pilot evidence.</x:v>
+      </x:c>
+      <x:c r="H69" s="50" t="str">
+        <x:v>Accountability practice: converts system failures into auditable methods, training, paid services, and institutional repair tools.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="70">
+      <x:c r="A70" s="51" t="str">
+        <x:v>The Batman Training Protocol and Productivity System</x:v>
+      </x:c>
+      <x:c r="B70" s="51" t="str">
+        <x:v>Consumer fitness and productivity planner</x:v>
+      </x:c>
+      <x:c r="C70" s="51" t="str">
+        <x:v>Rights-restricted draft; renamed original system after safety review</x:v>
+      </x:c>
+      <x:c r="D70" s="51" t="str">
+        <x:v>No match in recovered 60</x:v>
+      </x:c>
+      <x:c r="E70" s="51" t="str">
+        <x:v>Themed weekly conditioning schedule, productivity protocols, and readiness checklist combining exercise, logging, environment, reminders, and minimum progress.</x:v>
+      </x:c>
+      <x:c r="F70" s="51" t="str">
+        <x:v>Remove protected marks; progressive levels/rest/screening/injury modification; eliminate unsafe assumptions; trainer, sports-medicine, accessibility, rights review.</x:v>
+      </x:c>
+      <x:c r="G70" s="51" t="str">
+        <x:v>Rights-cleared workbook, facilitator kit, cohort course, institutional license, or consulting package after review and pilot evidence.</x:v>
+      </x:c>
+      <x:c r="H70" s="51" t="str">
+        <x:v>Audience and revenue: funds the mission, teaches the framework, and builds trust through useful rights-cleared products.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0688e04038b64e6a"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf53a884a4bb84902"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>